<commit_message>
camaraX grabacion a 1080 y copia a 720
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -13,11 +13,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.00 €"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -1715,7 +1716,7 @@
       </c>
       <c r="K5" s="58" t="inlineStr">
         <is>
-          <t>BC-7, BC-8</t>
+          <t>BC-7, BC-8, BC-9</t>
         </is>
       </c>
       <c r="L5" s="0">
@@ -1723,7 +1724,7 @@
         <v/>
       </c>
       <c r="M5" s="0" t="n">
-        <v>2425</v>
+        <v>3052</v>
       </c>
       <c r="N5" s="0">
         <f>SUMIFS($D$4:$D$29,$B$4:$B$29,"BC",$G$4:$G$29,"&lt;&gt;Sí")</f>
@@ -1778,7 +1779,7 @@
       </c>
       <c r="K6" s="58" t="inlineStr">
         <is>
-          <t>AN-2, AN-3, AN-4, AN-5</t>
+          <t>AN-2, AN-3, AN-4, AN-5, AN-6</t>
         </is>
       </c>
       <c r="L6" s="0">
@@ -1786,7 +1787,7 @@
         <v/>
       </c>
       <c r="M6" s="0" t="n">
-        <v>8177</v>
+        <v>10658</v>
       </c>
       <c r="N6" s="0">
         <f>SUMIFS($D$4:$D$29,$B$4:$B$29,"AN",$G$4:$G$29,"&lt;&gt;Sí")</f>
@@ -2254,6 +2255,302 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="57" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B19" s="58" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C19" s="58" t="inlineStr">
+        <is>
+          <t>BC-8</t>
+        </is>
+      </c>
+      <c r="D19" s="58" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E19" s="58" t="inlineStr">
+        <is>
+          <t>Senal sonora del PTT en la unidad: cinco tonos sintetizados en PCM con AudioTrack (subida al abrir, bajada al cerrar, zumbido si no se abre, y dos de recepcion), sonando en los seis puntos donde el PTT cambia de estado de verdad. Incluye el fallo por captura no confirmada del 8-sep, en el que el agente hablaba creyendo que le oian. Compila; sin oirse en la unidad</t>
+        </is>
+      </c>
+      <c r="F19" s="58" t="inlineStr">
+        <is>
+          <t>c000b50</t>
+        </is>
+      </c>
+      <c r="G19" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="58" t="inlineStr">
+        <is>
+          <t>marcas de fichero 08:41-12:21 (total medido; reparto por tarea estimado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="57" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B20" s="58" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C20" s="58" t="inlineStr">
+        <is>
+          <t>AN-4</t>
+        </is>
+      </c>
+      <c r="D20" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="58" t="inlineStr">
+        <is>
+          <t>Los mismos cinco tonos en el telefono (PttTones vive duplicado, como EvidenceCrypto) y los de recepcion cableados al PTT de un companero y al de la bodycam. Dos reglas que fijan el diseno: dos notas son tuyas y una nota es de otro, y el tono suena en el FLANCO y no en cada aviso de Agora. Compila; sin probar en aparatos</t>
+        </is>
+      </c>
+      <c r="F20" s="58" t="inlineStr">
+        <is>
+          <t>5492a2c</t>
+        </is>
+      </c>
+      <c r="G20" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="58" t="inlineStr">
+        <is>
+          <t>marcas de fichero 08:41-12:21 (total medido; reparto por tarea estimado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="57" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B21" s="58" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C21" s="58" t="inlineStr">
+        <is>
+          <t>AN-4</t>
+        </is>
+      </c>
+      <c r="D21" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="58" t="inlineStr">
+        <is>
+          <t>Recibir el PTT con la app cerrada: foreground service de tipo specialUse (mediaPlayback no se puede arrancar desde BOOT_COMPLETED con targetSdk 35+), atado al estado de sesion porque un telefono en el canal sin PIN es lo que prohibe el workflow 34; notificacion que dice quien esta hablando, BootReceiver y permiso de notificaciones. Compila; sin probar en aparatos</t>
+        </is>
+      </c>
+      <c r="F21" s="58" t="inlineStr">
+        <is>
+          <t>5492a2c</t>
+        </is>
+      </c>
+      <c r="G21" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H21" s="58" t="inlineStr">
+        <is>
+          <t>marcas de fichero 08:41-12:21 (total medido; reparto por tarea estimado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" s="38">
+      <c r="A22" s="57" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B22" s="58" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C22" s="58" t="inlineStr">
+        <is>
+          <t>AN-5</t>
+        </is>
+      </c>
+      <c r="D22" s="58" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E22" s="58" t="inlineStr">
+        <is>
+          <t>Armazon del video de las gafas: cliente HTTP contra 192.168.43.1 con los sockets atados a SU punto de acceso (nada de bindProcessToNetwork, que dejaria a Agora, subidas y mapa sin red) y descarga directa a la boveda cifrada, sin pasar por la galeria. Los tres datos del protocolo quedan marcados y NO inventados: hacen falta las gafas y una captura de trafico</t>
+        </is>
+      </c>
+      <c r="F22" s="58" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G22" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H22" s="58" t="inlineStr">
+        <is>
+          <t>marcas de fichero 08:41-12:21 (total medido; reparto por tarea estimado)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="57" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B23" s="58" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C23" s="58" t="n"/>
+      <c r="D23" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="58" t="inlineStr">
+        <is>
+          <t>Reunion</t>
+        </is>
+      </c>
+      <c r="F23" s="58" t="n"/>
+      <c r="G23" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H23" s="58" t="inlineStr">
+        <is>
+          <t>indicado por el usuario</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" s="38">
+      <c r="A24" s="57" t="n">
+        <v>46274</v>
+      </c>
+      <c r="B24" s="58" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C24" s="58" t="inlineStr">
+        <is>
+          <t>AN-5</t>
+        </is>
+      </c>
+      <c r="D24" s="58" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E24" s="58" t="inlineStr">
+        <is>
+          <t>Gafas BleeqUp, el WiFi resuelto. Integracion del SDK que entrego el fabricante (AAR en app/libs, OkHttp y Gson declarados a mano porque un .aar no trae sus dependencias, regla -keep de R8 para que Gson siga leyendo su JSON en release) y protocolo sacado de su bytecode: endpoints de listado, descarga con Range y borrado. LA CAUSA DEL FALLO: el SDK mete el codigo de pais del telefono en la orden BLE y el AP de las gafas emite en el canal 149 (5745 MHz), no permitido en Europa, asi que con ES el firmware se niega; con CN o US enciende. Ademas las gafas NO se anuncian nunca por BLE, asi que el escaneo del propio SDK no puede encontrarlas y hay que entregarle el aparato emparejado. Verificado de punta a punta en el Samsung: AP encendido, telefono unido y listado real de video e imagenes contra https://192.168.43.1</t>
+        </is>
+      </c>
+      <c r="F24" s="58" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G24" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H24" s="58" t="inlineStr">
+        <is>
+          <t>reloj de sesion 21:05-22:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="57" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B25" s="58" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C25" s="58" t="inlineStr">
+        <is>
+          <t>AN-6</t>
+        </is>
+      </c>
+      <c r="D25" s="58" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E25" s="58" t="inlineStr">
+        <is>
+          <t>Video original + proxy y SOS en la nube (telefono). Peticion del manager: original a 1080p sin recomprimir y copia de 720p/15 para que el backend la procese con un LLM. Grabacion con CameraX dentro de la app (el intent de la camara del sistema no deja fijar resolucion), proxy con Media3 Transformer cifrado y borrado al entregarse, subida kind=proxy antes que el original y reanudable. SOS desde la camara: cierra la grabacion, cede la camara al livestream y la reanuda al cancelar; avisos sos/start, latido y stop al backend para Agora Cloud Recording. Especificacion para backend (docs/BACKEND-PROXY-AND-SOS.md). Fallo cazado probando: CameraX recortaba el video a 886x1920. Verificado en el Samsung: original 1920x1080 a 30 fps, proxy 1280x720 a 15 fps, enlace por hash y SOS completo contra stubs</t>
+        </is>
+      </c>
+      <c r="F25" s="58" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G25" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H25" s="58" t="inlineStr">
+        <is>
+          <t>reloj de sesion 14:26-16:30 (2,1 h medidas), redondeado al alza a 3 h por indicacion del usuario; reparto por app estimado</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="57" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B26" s="58" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C26" s="58" t="inlineStr">
+        <is>
+          <t>BC-9</t>
+        </is>
+      </c>
+      <c r="D26" s="58" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E26" s="58" t="inlineStr">
+        <is>
+          <t>Video original + proxy y SOS en la nube (bodycam). El original deja de recodificarse (hasta hoy el rotulo del oficial se quemaba en la evidencia sellada): remux sin tocar los frames. Grabacion a 1080p cuando la camara lo ofrece (la W1 da 1920x1088), proxy de 720/15 con el rotulo solo ahi, bloque proxy en el manifest, subida manifest-proxy-original y aviso del SOS al backend. Verificado en la W1: el MP4 subido es el que escribio la camara (mismo hash), proxy 1264x720 a 14,9 fps, SOS completo contra stubs. Medido: la W1 graba a ~24-25 fps a cualquier resolucion</t>
+        </is>
+      </c>
+      <c r="F26" s="58" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G26" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H26" s="58" t="inlineStr">
+        <is>
+          <t>reloj de sesion 14:26-16:30 (2,1 h medidas), redondeado al alza a 3 h por indicacion del usuario; reparto por app estimado</t>
+        </is>
+      </c>
+    </row>
     <row r="31">
       <c r="C31" s="43" t="inlineStr">
         <is>
@@ -2268,7 +2565,7 @@
     <row r="33" ht="58" customHeight="1" s="38">
       <c r="A33" s="61" t="inlineStr">
         <is>
-          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4 más el trabajo del 6 y del 8 todavía sin commitear).</t>
+          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
controles de gafas y videos procesados
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -13,12 +13,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="#,##0.00\ &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.00 €"/>
-    <numFmt numFmtId="168" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -1787,7 +1786,7 @@
         <v/>
       </c>
       <c r="M6" s="0" t="n">
-        <v>10658</v>
+        <v>11633</v>
       </c>
       <c r="N6" s="0">
         <f>SUMIFS($D$4:$D$29,$B$4:$B$29,"AN",$G$4:$G$29,"&lt;&gt;Sí")</f>
@@ -2513,7 +2512,7 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" s="38">
       <c r="A26" s="57" t="n">
         <v>46276</v>
       </c>
@@ -2548,6 +2547,44 @@
       <c r="H26" s="58" t="inlineStr">
         <is>
           <t>reloj de sesion 14:26-16:30 (2,1 h medidas), redondeado al alza a 3 h por indicacion del usuario; reparto por app estimado</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" s="38">
+      <c r="A27" s="57" t="n">
+        <v>46277</v>
+      </c>
+      <c r="B27" s="58" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C27" s="58" t="inlineStr">
+        <is>
+          <t>AN-5</t>
+        </is>
+      </c>
+      <c r="D27" s="58" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="58" t="inlineStr">
+        <is>
+          <t>Mando a distancia de las gafas BleeqUp desde Nexus: arrancar y parar la grabacion y hacer foto por BLE, que hasta hoy no se podia (la app solo miraba si estaban enlazadas). Canal de mando propio (GafasCommandRepository) sobre el GATT del fabricante, con el arranque del SDK y el puente al aparato emparejado extraidos a un solo sitio (GafasSdkPuente), pantalla FALCON LENS con estado de los dos enlaces, resolucion y espacio libre de la tarjeta, y segundo boton de aparato en Operations. El GATT se suelta al salir de la pantalla: si se queda abierto, Android reusa el enlace cacheado y las escrituras siguientes fallan. LIMITE DEL SDK, escrito en pantalla: no existe ninguna orden para preguntar si las gafas estan grabando, asi que el indicador es la ultima orden dada y no un hecho; si el agente usa el boton fisico, el telefono no se entera. COMPILA SIN WARNINGS, SIN PROBAR CONTRA LAS GAFAS: no habia aparatos por adb</t>
+        </is>
+      </c>
+      <c r="F27" s="58" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G27" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" s="58" t="inlineStr">
+        <is>
+          <t>indicado por el usuario</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2602,7 @@
     <row r="33" ht="58" customHeight="1" s="38">
       <c r="A33" s="61" t="inlineStr">
         <is>
-          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.</t>
+          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
estado sos con gafas
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -1778,7 +1778,7 @@
       </c>
       <c r="K6" s="58" t="inlineStr">
         <is>
-          <t>AN-2, AN-3, AN-4, AN-5, AN-6</t>
+          <t>AN-2, AN-3, AN-4, AN-5, AN-6, AN-7</t>
         </is>
       </c>
       <c r="L6" s="0">
@@ -1786,7 +1786,7 @@
         <v/>
       </c>
       <c r="M6" s="0" t="n">
-        <v>11633</v>
+        <v>12109</v>
       </c>
       <c r="N6" s="0">
         <f>SUMIFS($D$4:$D$29,$B$4:$B$29,"AN",$G$4:$G$29,"&lt;&gt;Sí")</f>
@@ -2447,20 +2447,20 @@
       </c>
       <c r="C24" s="58" t="inlineStr">
         <is>
-          <t>AN-5</t>
+          <t>AN-7</t>
         </is>
       </c>
       <c r="D24" s="58" t="n">
-        <v>1.3</v>
+        <v>3</v>
       </c>
       <c r="E24" s="58" t="inlineStr">
         <is>
-          <t>Gafas BleeqUp, el WiFi resuelto. Integracion del SDK que entrego el fabricante (AAR en app/libs, OkHttp y Gson declarados a mano porque un .aar no trae sus dependencias, regla -keep de R8 para que Gson siga leyendo su JSON en release) y protocolo sacado de su bytecode: endpoints de listado, descarga con Range y borrado. LA CAUSA DEL FALLO: el SDK mete el codigo de pais del telefono en la orden BLE y el AP de las gafas emite en el canal 149 (5745 MHz), no permitido en Europa, asi que con ES el firmware se niega; con CN o US enciende. Ademas las gafas NO se anuncian nunca por BLE, asi que el escaneo del propio SDK no puede encontrarlas y hay que entregarle el aparato emparejado. Verificado de punta a punta en el Samsung: AP encendido, telefono unido y listado real de video e imagenes contra https://192.168.43.1</t>
+          <t>Boveda, categorizacion en bruto: la evidencia que llega de un periferico (gafas, bodycam) entra SIN incidente y la coloca el agente despues. Tabla raw_evidence con su DAO y BD a v2, apartado PENDING CATEGORIZATION arriba de la boveda, y dialogo de categorizacion con clasificacion, incidente y etiqueta: el agente elige un incidente ya abierto o crea uno nuevo. Dos reglas de diseno: el incidente que se crea se fecha en la GRABACION y no en el momento de categorizar, y lo que no se categoriza se queda en bruto con su fecha, no se pierde ni se le inventa un incidente. SESION QUE FALTABA EN EL LIBRO, detectada el 13-sep.</t>
         </is>
       </c>
       <c r="F24" s="58" t="inlineStr">
         <is>
-          <t>sin commitear</t>
+          <t>22768a9</t>
         </is>
       </c>
       <c r="G24" s="58" t="inlineStr">
@@ -2470,13 +2470,13 @@
       </c>
       <c r="H24" s="58" t="inlineStr">
         <is>
-          <t>reloj de sesion 21:05-22:25</t>
+          <t>marcas de fichero 13:13-15:57 (2,7 h medidas), redondeado al alza a 3 h</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="57" t="n">
-        <v>46276</v>
+        <v>46274</v>
       </c>
       <c r="B25" s="58" t="inlineStr">
         <is>
@@ -2485,15 +2485,15 @@
       </c>
       <c r="C25" s="58" t="inlineStr">
         <is>
-          <t>AN-6</t>
+          <t>AN-5</t>
         </is>
       </c>
       <c r="D25" s="58" t="n">
-        <v>1.8</v>
+        <v>1.3</v>
       </c>
       <c r="E25" s="58" t="inlineStr">
         <is>
-          <t>Video original + proxy y SOS en la nube (telefono). Peticion del manager: original a 1080p sin recomprimir y copia de 720p/15 para que el backend la procese con un LLM. Grabacion con CameraX dentro de la app (el intent de la camara del sistema no deja fijar resolucion), proxy con Media3 Transformer cifrado y borrado al entregarse, subida kind=proxy antes que el original y reanudable. SOS desde la camara: cierra la grabacion, cede la camara al livestream y la reanuda al cancelar; avisos sos/start, latido y stop al backend para Agora Cloud Recording. Especificacion para backend (docs/BACKEND-PROXY-AND-SOS.md). Fallo cazado probando: CameraX recortaba el video a 886x1920. Verificado en el Samsung: original 1920x1080 a 30 fps, proxy 1280x720 a 15 fps, enlace por hash y SOS completo contra stubs</t>
+          <t>Gafas BleeqUp, el WiFi resuelto. Integracion del SDK que entrego el fabricante (AAR en app/libs, OkHttp y Gson declarados a mano porque un .aar no trae sus dependencias, regla -keep de R8 para que Gson siga leyendo su JSON en release) y protocolo sacado de su bytecode: endpoints de listado, descarga con Range y borrado. LA CAUSA DEL FALLO: el SDK mete el codigo de pais del telefono en la orden BLE y el AP de las gafas emite en el canal 149 (5745 MHz), no permitido en Europa, asi que con ES el firmware se niega; con CN o US enciende. Ademas las gafas NO se anuncian nunca por BLE, asi que el escaneo del propio SDK no puede encontrarlas y hay que entregarle el aparato emparejado. Verificado de punta a punta en el Samsung: AP encendido, telefono unido y listado real de video e imagenes contra https://192.168.43.1</t>
         </is>
       </c>
       <c r="F25" s="58" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="H25" s="58" t="inlineStr">
         <is>
-          <t>reloj de sesion 14:26-16:30 (2,1 h medidas), redondeado al alza a 3 h por indicacion del usuario; reparto por app estimado</t>
+          <t>reloj de sesion 21:05-22:25</t>
         </is>
       </c>
     </row>
@@ -2518,20 +2518,20 @@
       </c>
       <c r="B26" s="58" t="inlineStr">
         <is>
-          <t>BC</t>
+          <t>AN</t>
         </is>
       </c>
       <c r="C26" s="58" t="inlineStr">
         <is>
-          <t>BC-9</t>
+          <t>AN-6</t>
         </is>
       </c>
       <c r="D26" s="58" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="E26" s="58" t="inlineStr">
         <is>
-          <t>Video original + proxy y SOS en la nube (bodycam). El original deja de recodificarse (hasta hoy el rotulo del oficial se quemaba en la evidencia sellada): remux sin tocar los frames. Grabacion a 1080p cuando la camara lo ofrece (la W1 da 1920x1088), proxy de 720/15 con el rotulo solo ahi, bloque proxy en el manifest, subida manifest-proxy-original y aviso del SOS al backend. Verificado en la W1: el MP4 subido es el que escribio la camara (mismo hash), proxy 1264x720 a 14,9 fps, SOS completo contra stubs. Medido: la W1 graba a ~24-25 fps a cualquier resolucion</t>
+          <t>Video original + proxy y SOS en la nube (telefono). Peticion del manager: original a 1080p sin recomprimir y copia de 720p/15 para que el backend la procese con un LLM. Grabacion con CameraX dentro de la app (el intent de la camara del sistema no deja fijar resolucion), proxy con Media3 Transformer cifrado y borrado al entregarse, subida kind=proxy antes que el original y reanudable. SOS desde la camara: cierra la grabacion, cede la camara al livestream y la reanuda al cancelar; avisos sos/start, latido y stop al backend para Agora Cloud Recording. Especificacion para backend (docs/BACKEND-PROXY-AND-SOS.md). Fallo cazado probando: CameraX recortaba el video a 886x1920. Verificado en el Samsung: original 1920x1080 a 30 fps, proxy 1280x720 a 15 fps, enlace por hash y SOS completo contra stubs</t>
         </is>
       </c>
       <c r="F26" s="58" t="inlineStr">
@@ -2552,37 +2552,75 @@
     </row>
     <row r="27" s="38">
       <c r="A27" s="57" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B27" s="58" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C27" s="58" t="inlineStr">
+        <is>
+          <t>BC-9</t>
+        </is>
+      </c>
+      <c r="D27" s="58" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E27" s="58" t="inlineStr">
+        <is>
+          <t>Video original + proxy y SOS en la nube (bodycam). El original deja de recodificarse (hasta hoy el rotulo del oficial se quemaba en la evidencia sellada): remux sin tocar los frames. Grabacion a 1080p cuando la camara lo ofrece (la W1 da 1920x1088), proxy de 720/15 con el rotulo solo ahi, bloque proxy en el manifest, subida manifest-proxy-original y aviso del SOS al backend. Verificado en la W1: el MP4 subido es el que escribio la camara (mismo hash), proxy 1264x720 a 14,9 fps, SOS completo contra stubs. Medido: la W1 graba a ~24-25 fps a cualquier resolucion</t>
+        </is>
+      </c>
+      <c r="F27" s="58" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G27" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H27" s="58" t="inlineStr">
+        <is>
+          <t>reloj de sesion 14:26-16:30 (2,1 h medidas), redondeado al alza a 3 h por indicacion del usuario; reparto por app estimado</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="57" t="n">
         <v>46277</v>
       </c>
-      <c r="B27" s="58" t="inlineStr">
+      <c r="B28" s="58" t="inlineStr">
         <is>
           <t>AN</t>
         </is>
       </c>
-      <c r="C27" s="58" t="inlineStr">
+      <c r="C28" s="58" t="inlineStr">
         <is>
           <t>AN-5</t>
         </is>
       </c>
-      <c r="D27" s="58" t="n">
+      <c r="D28" s="58" t="n">
         <v>3</v>
       </c>
-      <c r="E27" s="58" t="inlineStr">
+      <c r="E28" s="58" t="inlineStr">
         <is>
           <t>Mando a distancia de las gafas BleeqUp desde Nexus: arrancar y parar la grabacion y hacer foto por BLE, que hasta hoy no se podia (la app solo miraba si estaban enlazadas). Canal de mando propio (GafasCommandRepository) sobre el GATT del fabricante, con el arranque del SDK y el puente al aparato emparejado extraidos a un solo sitio (GafasSdkPuente), pantalla FALCON LENS con estado de los dos enlaces, resolucion y espacio libre de la tarjeta, y segundo boton de aparato en Operations. El GATT se suelta al salir de la pantalla: si se queda abierto, Android reusa el enlace cacheado y las escrituras siguientes fallan. LIMITE DEL SDK, escrito en pantalla: no existe ninguna orden para preguntar si las gafas estan grabando, asi que el indicador es la ultima orden dada y no un hecho; si el agente usa el boton fisico, el telefono no se entera. COMPILA SIN WARNINGS, SIN PROBAR CONTRA LAS GAFAS: no habia aparatos por adb</t>
         </is>
       </c>
-      <c r="F27" s="58" t="inlineStr">
+      <c r="F28" s="58" t="inlineStr">
         <is>
           <t>sin commitear</t>
         </is>
       </c>
-      <c r="G27" s="58" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="H27" s="58" t="inlineStr">
+      <c r="G28" s="58" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H28" s="58" t="inlineStr">
         <is>
           <t>indicado por el usuario</t>
         </is>
@@ -2602,7 +2640,7 @@
     <row r="33" ht="58" customHeight="1" s="38">
       <c r="A33" s="61" t="inlineStr">
         <is>
-          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.</t>
+          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
agora repositorio arreglado con ptt
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -17212,14 +17212,14 @@
         </is>
       </c>
       <c r="L5" s="13">
-        <f>SUMPRODUCT(($B$4:$B$33="BC")/COUNTIFS($A$4:$A$33,$A$4:$A$33&amp;"",$B$4:$B$33,$B$4:$B$33&amp;""))</f>
+        <f>SUMPRODUCT(($B$4:$B$43="BC")/COUNTIFS($A$4:$A$43,$A$4:$A$43&amp;"",$B$4:$B$43,$B$4:$B$43&amp;""))</f>
         <v/>
       </c>
       <c r="M5" s="13" t="n">
-        <v>3343</v>
+        <v>3651</v>
       </c>
       <c r="N5" s="13">
-        <f>SUMIFS($D$4:$D$33,$B$4:$B$33,"BC",$G$4:$G$33,"&lt;&gt;Sí")</f>
+        <f>SUMIFS($D$4:$D$43,$B$4:$B$43,"BC",$G$4:$G$43,"&lt;&gt;Sí")</f>
         <v/>
       </c>
       <c r="O5" s="9">
@@ -17275,14 +17275,14 @@
         </is>
       </c>
       <c r="L6" s="13">
-        <f>SUMPRODUCT(($B$4:$B$33="AN")/COUNTIFS($A$4:$A$33,$A$4:$A$33&amp;"",$B$4:$B$33,$B$4:$B$33&amp;""))</f>
+        <f>SUMPRODUCT(($B$4:$B$43="AN")/COUNTIFS($A$4:$A$43,$A$4:$A$43&amp;"",$B$4:$B$43,$B$4:$B$43&amp;""))</f>
         <v/>
       </c>
       <c r="M6" s="13" t="n">
-        <v>15629</v>
+        <v>15651</v>
       </c>
       <c r="N6" s="13">
-        <f>SUMIFS($D$4:$D$33,$B$4:$B$33,"AN",$G$4:$G$33,"&lt;&gt;Sí")</f>
+        <f>SUMIFS($D$4:$D$43,$B$4:$B$43,"AN",$G$4:$G$43,"&lt;&gt;Sí")</f>
         <v/>
       </c>
       <c r="O6" s="9">
@@ -17329,11 +17329,11 @@
         </is>
       </c>
       <c r="K7" s="13">
-        <f>SUMPRODUCT(($C$4:$C$33&lt;&gt;"")/COUNTIF($C$4:$C$33,$C$4:$C$33&amp;""))</f>
+        <f>SUMPRODUCT(($C$4:$C$43&lt;&gt;"")/COUNTIF($C$4:$C$43,$C$4:$C$43&amp;""))</f>
         <v/>
       </c>
       <c r="L7" s="13">
-        <f>SUMPRODUCT(($A$4:$A$33&lt;&gt;"")/COUNTIF($A$4:$A$33,$A$4:$A$33&amp;""))</f>
+        <f>SUMPRODUCT(($A$4:$A$43&lt;&gt;"")/COUNTIF($A$4:$A$43,$A$4:$A$43&amp;""))</f>
         <v/>
       </c>
       <c r="M7" s="10">
@@ -18420,14 +18420,42 @@
       <c r="O32" s="2" t="n"/>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="15">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
-      <c r="H33" s="11" t="n"/>
+      <c r="A33" s="6" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>AN-4</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>PTT del telefono como conmutador (peticion del usuario): un toque abre el canal y otro lo cierra, en lugar de mantener pulsado; se sigue cerrando al salir de Operations y, al conceder el permiso de microfono, el canal se abre sin repetir el toque. Diagnostico de por que el PTT del Samsung no llegaba a nadie: llevaba fuera del canal desde la 01:44 (Agora dio la conexion por fallida tras 20 min sin red), Nexus no vuelve a entrar y sigue marcando ONLINE. Fallo documentado, SIN ARREGLAR. Verificado en el Samsung: micro abierto 13:03:32 y cerrado 13:03:39 con dos toques</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>reloj de sesion 12:28-13:07 (0,65 h medidas), redondeado al alza a 1 h; reparto por app estimado sobre las marcas de fichero</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="n"/>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="n"/>
@@ -18436,21 +18464,42 @@
       <c r="O33" s="2" t="n"/>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="15">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="10" t="inlineStr">
+      <c r="A34" s="6" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>TOTAL HORAS</t>
+          <t>BC</t>
         </is>
       </c>
-      <c r="D34" s="10">
-        <f>SUM($D$4:$D$33)</f>
-        <v/>
-      </c>
-      <c r="E34" s="2" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>BC-8</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>PTT del telefono sonando en la bodycam, punto 1: la W1 esta siempre en el canal de Agora como audiencia, sin capturar, con un solo motor compartido. El SOS y el PTT de la unidad ya no entran ni salen del canal: suben a emitir y vuelven a escuchar. Reentrada tras perder la conexion y SOS pedido sin red que sale al volver. Verificado en la W1: entra en 333 ms, la grabacion conserva el microfono, PTT y SOS propios suben y bajan y rearman el anillo, y el PTT del Samsung se reproduce en la unidad (DECODING)</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>reloj de sesion 12:28-13:07 (0,65 h medidas), redondeado al alza a 1 h; reparto por app estimado sobre las marcas de fichero</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="n"/>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
@@ -18459,14 +18508,14 @@
       <c r="O34" s="2" t="n"/>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="15">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="2" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
+      <c r="A35" s="6" t="n"/>
+      <c r="B35" s="11" t="n"/>
+      <c r="C35" s="11" t="n"/>
+      <c r="D35" s="11" t="n"/>
+      <c r="E35" s="11" t="n"/>
+      <c r="F35" s="11" t="n"/>
+      <c r="G35" s="11" t="n"/>
+      <c r="H35" s="11" t="n"/>
       <c r="J35" s="2" t="n"/>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="n"/>
@@ -18474,12 +18523,15 @@
       <c r="N35" s="2" t="n"/>
       <c r="O35" s="2" t="n"/>
     </row>
-    <row r="36" ht="57.75" customHeight="1" s="15">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.    RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33; el total paso a la fila 34 y esta leyenda a la 36. La fila 33 es la ultima libre: para seguir hay que volver a ampliar.</t>
-        </is>
-      </c>
+    <row r="36" ht="15.75" customHeight="1" s="15">
+      <c r="A36" s="6" t="n"/>
+      <c r="B36" s="11" t="n"/>
+      <c r="C36" s="11" t="n"/>
+      <c r="D36" s="11" t="n"/>
+      <c r="E36" s="11" t="n"/>
+      <c r="F36" s="11" t="n"/>
+      <c r="G36" s="11" t="n"/>
+      <c r="H36" s="11" t="n"/>
       <c r="J36" s="2" t="n"/>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
@@ -18488,14 +18540,14 @@
       <c r="O36" s="2" t="n"/>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="15">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
+      <c r="A37" s="6" t="n"/>
+      <c r="B37" s="11" t="n"/>
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="11" t="n"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+      <c r="H37" s="11" t="n"/>
       <c r="J37" s="2" t="n"/>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="n"/>
@@ -18504,14 +18556,14 @@
       <c r="O37" s="2" t="n"/>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="15">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="11" t="n"/>
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="11" t="n"/>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="11" t="n"/>
       <c r="J38" s="2" t="n"/>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="n"/>
@@ -18520,14 +18572,14 @@
       <c r="O38" s="2" t="n"/>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="15">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="2" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
+      <c r="A39" s="6" t="n"/>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="11" t="n"/>
       <c r="J39" s="2" t="n"/>
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="n"/>
@@ -18536,14 +18588,14 @@
       <c r="O39" s="2" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="15">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="2" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
+      <c r="A40" s="6" t="n"/>
+      <c r="B40" s="11" t="n"/>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="11" t="n"/>
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="11" t="n"/>
       <c r="J40" s="2" t="n"/>
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="n"/>
@@ -18552,14 +18604,14 @@
       <c r="O40" s="2" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="15">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="2" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
+      <c r="A41" s="6" t="n"/>
+      <c r="B41" s="11" t="n"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="11" t="n"/>
+      <c r="E41" s="11" t="n"/>
+      <c r="F41" s="11" t="n"/>
+      <c r="G41" s="11" t="n"/>
+      <c r="H41" s="11" t="n"/>
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="n"/>
@@ -18568,14 +18620,14 @@
       <c r="O41" s="2" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="15">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="2" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
+      <c r="A42" s="6" t="n"/>
+      <c r="B42" s="11" t="n"/>
+      <c r="C42" s="11" t="n"/>
+      <c r="D42" s="11" t="n"/>
+      <c r="E42" s="11" t="n"/>
+      <c r="F42" s="11" t="n"/>
+      <c r="G42" s="11" t="n"/>
+      <c r="H42" s="11" t="n"/>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="n"/>
@@ -18584,14 +18636,14 @@
       <c r="O42" s="2" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="15">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
+      <c r="A43" s="6" t="n"/>
+      <c r="B43" s="11" t="n"/>
+      <c r="C43" s="11" t="n"/>
+      <c r="D43" s="11" t="n"/>
+      <c r="E43" s="11" t="n"/>
+      <c r="F43" s="11" t="n"/>
+      <c r="G43" s="11" t="n"/>
+      <c r="H43" s="11" t="n"/>
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
@@ -18602,8 +18654,15 @@
     <row r="44" ht="15.75" customHeight="1" s="15">
       <c r="A44" s="2" t="n"/>
       <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
+      <c r="C44" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL HORAS</t>
+        </is>
+      </c>
+      <c r="D44" s="10">
+        <f>SUM($D$4:$D$43)</f>
+        <v/>
+      </c>
       <c r="E44" s="2" t="n"/>
       <c r="F44" s="2" t="n"/>
       <c r="G44" s="2" t="n"/>
@@ -18631,15 +18690,12 @@
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="2" t="n"/>
     </row>
-    <row r="46" ht="15.75" customHeight="1" s="15">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="2" t="n"/>
-      <c r="F46" s="2" t="n"/>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
+    <row r="46" ht="57.75" customHeight="1" s="15">
+      <c r="A46" s="14" t="inlineStr">
+        <is>
+          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.   15 DE SEPTIEMBRE: AN-4 y BC-8 (PTT). BC-8 = la bodycam escucha el canal todo el tiempo para que el PTT de los telefonos suene por su altavoz (punto 1 de los requisitos del 14-sep). AN-4 = boton de PTT del telefono de un toque, y diagnostico de que Nexus no vuelve al canal tras perder la conexion (documentado, sin arreglar). Las horas salen del reloj de sesion 12:28-13:07 (0,65 h medidas), redondeadas al alza a 1 h; el reparto 0,5 / 0,5 es estimacion sobre las marcas de fichero (BodyCamServer 12:34-12:49, Nexus 12:59-13:04). Lineas del 15, sin commitear, medidas con git: 308 anadidas en BC (de ellas 279 en LivestreamService, reescrito: salen tambien 216) y 22 en AN.   RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33 y el 15-sep a la 43; el total esta en la fila 44 y esta leyenda en la 46. Ultima fila libre: la 43.</t>
+        </is>
+      </c>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
@@ -33913,7 +33969,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>

</xml_diff>

<commit_message>
previo a conectar con backend
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -17216,7 +17216,7 @@
         <v/>
       </c>
       <c r="M5" s="13" t="n">
-        <v>3651</v>
+        <v>3662</v>
       </c>
       <c r="N5" s="13">
         <f>SUMIFS($D$4:$D$43,$B$4:$B$43,"BC",$G$4:$G$43,"&lt;&gt;Sí")</f>
@@ -17279,7 +17279,7 @@
         <v/>
       </c>
       <c r="M6" s="13" t="n">
-        <v>17637</v>
+        <v>17763</v>
       </c>
       <c r="N6" s="13">
         <f>SUMIFS($D$4:$D$43,$B$4:$B$43,"AN",$G$4:$G$43,"&lt;&gt;Sí")</f>
@@ -17323,29 +17323,29 @@
           <t>reloj de sesion 16:19-20:42 (total medido; reparto por tarea estimado)</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr">
-        <is>
-          <t>TOTAL DEL MES</t>
-        </is>
-      </c>
-      <c r="K7" s="13">
-        <f>SUMPRODUCT(($C$4:$C$43&lt;&gt;"")/COUNTIF($C$4:$C$43,$C$4:$C$43&amp;""))</f>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>aeria-nexus (backend)</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>NX-1, NX-2, NX-3</t>
+        </is>
+      </c>
+      <c r="L7" s="13">
+        <f>SUMPRODUCT(($B$4:$B$43="NX")/COUNTIFS($A$4:$A$43,$A$4:$A$43&amp;"",$B$4:$B$43,$B$4:$B$43&amp;""))</f>
         <v/>
       </c>
-      <c r="L7" s="13">
-        <f>SUMPRODUCT(($A$4:$A$43&lt;&gt;"")/COUNTIF($A$4:$A$43,$A$4:$A$43&amp;""))</f>
+      <c r="M7" s="13" t="n">
+        <v>10475</v>
+      </c>
+      <c r="N7" s="13">
+        <f>SUMIFS($D$4:$D$43,$B$4:$B$43,"NX",$G$4:$G$43,"&lt;&gt;Sí")</f>
         <v/>
       </c>
-      <c r="M7" s="10">
-        <f>SUM(M5:M6)</f>
-        <v/>
-      </c>
-      <c r="N7" s="10">
-        <f>SUM(N5:N6)</f>
-        <v/>
-      </c>
-      <c r="O7" s="12">
-        <f>SUM(O5:O6)</f>
+      <c r="O7" s="9">
+        <f>N7*$K$9</f>
         <v/>
       </c>
     </row>
@@ -17382,12 +17382,31 @@
           <t>reloj de sesion 16:19-20:42 (total medido; reparto por tarea estimado)</t>
         </is>
       </c>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="n"/>
-      <c r="O8" s="2" t="n"/>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>TOTAL DEL MES</t>
+        </is>
+      </c>
+      <c r="K8" s="13">
+        <f>SUMPRODUCT(($C$4:$C$43&lt;&gt;"")/COUNTIF($C$4:$C$43,$C$4:$C$43&amp;""))</f>
+        <v/>
+      </c>
+      <c r="L8" s="13">
+        <f>SUMPRODUCT(($A$4:$A$43&lt;&gt;"")/COUNTIF($A$4:$A$43,$A$4:$A$43&amp;""))</f>
+        <v/>
+      </c>
+      <c r="M8" s="10">
+        <f>SUM(M5:M7)</f>
+        <v/>
+      </c>
+      <c r="N8" s="10">
+        <f>SUM(N5:N7)</f>
+        <v/>
+      </c>
+      <c r="O8" s="12">
+        <f>SUM(O5:O7)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -18728,14 +18747,42 @@
       <c r="O39" s="2" t="n"/>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="15">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="11" t="n"/>
-      <c r="C40" s="11" t="n"/>
-      <c r="D40" s="11" t="n"/>
-      <c r="E40" s="11" t="n"/>
-      <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
-      <c r="H40" s="11" t="n"/>
+      <c r="A40" s="6" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>AN-4</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>PTT pisado (peticion del usuario): si un agente esta hablando con el PTT abierto y otro abre el suyo encima, o al reves, suena un tono nuevo de tres pitidos agudos a volumen pleno (el pitido normal de recepcion quedaba tapado por la propia voz) y el boton PTT se pone ambar con icono de aviso y '&lt;oficial&gt; ALSO ON AIR'. Cuenta tambien la bodycam del propio agente. Tono copiado igual en BodyCamServer para mantener los tonos gemelos. Atajo debug para simular el PTT de otro agente con un solo telefono. Verificado en el Samsung con ese atajo (pantalla y numero de tonos en los cuatro casos); falta la prueba con dos telefonos reales.</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>indicado por el usuario: 1 h</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="n"/>
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="n"/>
@@ -18744,14 +18791,42 @@
       <c r="O40" s="2" t="n"/>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="15">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="11" t="n"/>
-      <c r="C41" s="11" t="n"/>
-      <c r="D41" s="11" t="n"/>
-      <c r="E41" s="11" t="n"/>
-      <c r="F41" s="11" t="n"/>
-      <c r="G41" s="11" t="n"/>
-      <c r="H41" s="11" t="n"/>
+      <c r="A41" s="6" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>NX-1</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>Backend, arranque del ecosistema e identidad: repositorio de contratos aeria-contracts (upload-protocol, crypto-format, manifest-schema, iam-session, insights-schema, openapi) y simulador de cliente que recorre enrolamiento, sesion y las tres subidas generando un .fev real; tres costuras de portabilidad (almacen de evidencia, desenvoltura de claves, esquema de insights) para que ningun otro sitio hable con el SDK de un proveedor; e IAM F1-F6: modelos de identidad, dos CA separadas, enrolamiento de dispositivo y de agente con CSR y prueba de posesion, retos y sesion por token, autorizacion por rol con acotado de la evidencia, login del panel por persona y revocacion. 229 tests</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>fc48ce9, ebc20a7, 970b5df, b0b8734, dd2998d, e2e6924, 472c800</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>commits 15:32-18:47 (3,25 h medidas, al alza 3,5 segun la regla del 13-sep)</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="n"/>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="n"/>
@@ -18760,14 +18835,42 @@
       <c r="O41" s="2" t="n"/>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="15">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="11" t="n"/>
-      <c r="C42" s="11" t="n"/>
-      <c r="D42" s="11" t="n"/>
-      <c r="E42" s="11" t="n"/>
-      <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
-      <c r="H42" s="11" t="n"/>
+      <c r="A42" s="6" t="n">
+        <v>46281</v>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>NX-2</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>Backend, ingesta de evidencia y analisis: endpoint tus 1.0.0 reanudable con verificacion de integridad por sha256 del cifrado; y enlace subida-&gt;analisis, que era la cadena rota (recuperar del almacen, descifrar el .fev, temporal en claro que se borra pase lo que pase, verificacion de custodia contra el sha256_plain del manifiesto, mapeo al esquema canonico y encolado automatico). Tres fallos propios encontrados al probar: descriptor de mkstemp sin cerrar, try que no protegia el on_commit, y 109 s de espera al encolar sin Redis por el almacen de resultados. 250 tests</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>ec1d5cf, 8115e2c, 6cc9451</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>commits 18:47-23:42 (4,9 h medidas, al alza 5)</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="n"/>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="n"/>
@@ -18776,14 +18879,42 @@
       <c r="O42" s="2" t="n"/>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="15">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="11" t="n"/>
-      <c r="C43" s="11" t="n"/>
-      <c r="D43" s="11" t="n"/>
-      <c r="E43" s="11" t="n"/>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
+      <c r="A43" s="6" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>NX-3</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Backend, coste medido y demostracion: modelo de coste con las tarifas reales aportadas por el usuario, midiendo los ocho prompts en el codigo (0,45 EUR por incidente de 10 min; el indexador cuesta 3,5 veces el modelo, al reves de lo que decia la documentacion). Dos fallos propios del dia anterior arreglados (NameError en init_conversation y json.dumps sobre un dataclass, que colaba un repr de Python en el prompt) y cerrado el test de login intermitente parando el reloj. Comando inspeccionar_subidas para ver que llega de verdad de un dispositivo, abriendo el sobre cifrado. Y descubierto y arreglado que el panel no podia reproducir NINGUN video subido por un agente: modulo preview con descifrado a copia reutilizable, mas interruptor para apagar el indicador de IA en la demostracion. 264 tests</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>2,5 h indicadas por el usuario; la sesion se prolongo pasada la medianoche y se imputa entera al 17</t>
+        </is>
+      </c>
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
@@ -18833,7 +18964,7 @@
     <row r="46" ht="57.75" customHeight="1" s="15">
       <c r="A46" s="14" t="inlineStr">
         <is>
-          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.   15 DE SEPTIEMBRE: AN-4 y BC-8 (PTT). BC-8 = la bodycam escucha el canal todo el tiempo para que el PTT de los telefonos suene por su altavoz (punto 1 de los requisitos del 14-sep). AN-4 = boton de PTT del telefono de un toque, y diagnostico de que Nexus no vuelve al canal tras perder la conexion (documentado, sin arreglar). Las horas salen del reloj de sesion 12:28-13:07 (0,65 h medidas), redondeadas al alza a 1 h; el reparto 0,5 / 0,5 es estimacion sobre las marcas de fichero (BodyCamServer 12:34-12:49, Nexus 12:59-13:04). Lineas del 15, sin commitear, medidas con git: 308 anadidas en BC (de ellas 279 en LivestreamService, reescrito: salen tambien 216) y 22 en AN.   15 DE SEPTIEMBRE, TARDE: AN-4 = reconexion al canal de Agora (el telefono se quedaba fuera sin avisar). AN-2 = revision del IAM y workflows 5 (cambio de PIN) y 30 (fin de turno). AN-10 (bloque nuevo) = auditoria local, workflows 61 y 46. Las horas salen del reloj de sesion 13:34-14:05 y 14:22-15:06 (1,25 h medidas), redondeadas al alza a 1,5 h; el reparto 0,3 / 0,6 / 0,6 es estimacion sobre la hora de cada peticion. NO se cuentan 13:20-13:34, que fue anotar en esta tabla las horas de la manana, ni 14:05-14:22, espera a que se desbloqueara el telefono de pruebas. Lineas .kt: 176 de la reconexion (commit 49d8c20, sin las 22 del boton de PTT ya contadas en la fila 33); unas 529 de los wf 5 y 30 y unas 903 de los wf 61 y 46, de ellas 96 de pruebas JVM, sin commitear; el reparto entre bloques de los ficheros compartidos (IdentityRepository, ProfileScreen, AppNavHost, AppContainer) es estimacion.   15 DE SEPTIEMBRE, FINAL DE LA TARDE: AN-5 (gafas) = selector de gafas sin MAC compilada, y arreglo de la conexion en Android 11 (el SDK del fabricante comprobaba un permiso que en esa version no existe). Las 2 h las indico el usuario; la sesion registra 0,85 h activas (15:06-15:27, 16:03-16:26 y 16:41-16:48) y los huecos 15:27-16:03 y 16:26-16:41 fueron del usuario con la release del manager y las pruebas en el Redmi. Reparto 1 / 1 estimado. Lineas .kt sin commitear, medidas con git: 378 (unas 343 del selector y unas 35 del arreglo de Android 11).   RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33 y el 15-sep a la 43; el total esta en la fila 44 y esta leyenda en la 46. Ultima fila libre: la 43.</t>
+          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.   15 DE SEPTIEMBRE: AN-4 y BC-8 (PTT). BC-8 = la bodycam escucha el canal todo el tiempo para que el PTT de los telefonos suene por su altavoz (punto 1 de los requisitos del 14-sep). AN-4 = boton de PTT del telefono de un toque, y diagnostico de que Nexus no vuelve al canal tras perder la conexion (documentado, sin arreglar). Las horas salen del reloj de sesion 12:28-13:07 (0,65 h medidas), redondeadas al alza a 1 h; el reparto 0,5 / 0,5 es estimacion sobre las marcas de fichero (BodyCamServer 12:34-12:49, Nexus 12:59-13:04). Lineas del 15, sin commitear, medidas con git: 308 anadidas en BC (de ellas 279 en LivestreamService, reescrito: salen tambien 216) y 22 en AN.   15 DE SEPTIEMBRE, TARDE: AN-4 = reconexion al canal de Agora (el telefono se quedaba fuera sin avisar). AN-2 = revision del IAM y workflows 5 (cambio de PIN) y 30 (fin de turno). AN-10 (bloque nuevo) = auditoria local, workflows 61 y 46. Las horas salen del reloj de sesion 13:34-14:05 y 14:22-15:06 (1,25 h medidas), redondeadas al alza a 1,5 h; el reparto 0,3 / 0,6 / 0,6 es estimacion sobre la hora de cada peticion. NO se cuentan 13:20-13:34, que fue anotar en esta tabla las horas de la manana, ni 14:05-14:22, espera a que se desbloqueara el telefono de pruebas. Lineas .kt: 176 de la reconexion (commit 49d8c20, sin las 22 del boton de PTT ya contadas en la fila 33); unas 529 de los wf 5 y 30 y unas 903 de los wf 61 y 46, de ellas 96 de pruebas JVM, sin commitear; el reparto entre bloques de los ficheros compartidos (IdentityRepository, ProfileScreen, AppNavHost, AppContainer) es estimacion.   15 DE SEPTIEMBRE, FINAL DE LA TARDE: AN-5 (gafas) = selector de gafas sin MAC compilada, y arreglo de la conexion en Android 11 (el SDK del fabricante comprobaba un permiso que en esa version no existe). Las 2 h las indico el usuario; la sesion registra 0,85 h activas (15:06-15:27, 16:03-16:26 y 16:41-16:48) y los huecos 15:27-16:03 y 16:26-16:41 fueron del usuario con la release del manager y las pruebas en el Redmi. Reparto 1 / 1 estimado. Lineas .kt sin commitear, medidas con git: 378 (unas 343 del selector y unas 35 del arreglo de Android 11).   15 DE SEPTIEMBRE, NOCHE: AN-4 (PTT) = aviso de PTT pisado, con tono de tres pitidos y boton ambar cuando dos agentes hablan a la vez. La hora la indico el usuario. Lineas .kt sin commitear, medidas con git: 126 en AN (19 del atajo de debug) y 11 en BC (el tono gemelo en PttTones).   RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33 y el 15-sep a la 43; el total esta en la fila 44 y esta leyenda en la 46. RANGO AGOTADO: las filas 41, 42 y 43 se ocuparon el 17-sep con el backend. NO QUEDA NINGUNA FILA LIBRE: la proxima sesion tiene que ampliar el rango de las formulas (D44 y las seis de las filas 5 a 8) y bajar el total y esta leyenda, como se hizo el 14 y el 15 de septiembre.   16 Y 17 DE SEPTIEMBRE, BACKEND (aplicacion NX, nueva): NX es el tercer repositorio, aeria-nexus, que hasta hoy no estaba en este libro aunque llevaba dos dias de trabajo. Django 5 + DRF + Celery y el panel Next.js, mas el repositorio de contratos aeria-contracts, que se imputa aqui porque nacio dentro de estas mismas sesiones. NX-1 = contratos, simulador de cliente, costuras de portabilidad e identidad F1-F6. NX-2 = ingesta de evidencia por tus y enlace de la subida con el analisis. NX-3 = coste medido, arreglos y puesta a punto para la demostracion al manager.   ORIGEN DE LAS HORAS DEL BACKEND: las dos filas del 16 salen de las marcas de los commits, 15:32 (primer commit de contratos) a 23:42 (ultimo del backend), 8,15 h medidas; el corte entre NX-1 y NX-2 es el commit de las 18:47, que cierra identidad. Cada tramo se redondea al alza al medio punto por separado (3,25-&gt;3,5 y 4,9-&gt;5), asi que la suma imputada del dia es 8,5. NO se cuenta nada anterior al primer commit. Las 2,5 h del 17 las indico el usuario: esa sesion no dejo commits, se prolongo pasada la medianoche y se imputa entera al 17.   LINEAS DE CODIGO DEL BACKEND: 10.475, medidas con git y contando solo codigo (.py, .ts, .tsx). Del 16 son 9.871 en diez commits; del 17, 604 sin commitear (469 de cuatro ficheros nuevos y 135 de modificaciones). NO se cuentan 2.210 lineas de documentacion en Markdown de los dos dias, ni las 1.028 del simulador de cliente y 456 del OpenAPI que viven en aeria-contracts, aunque se escribieran en estas sesiones: quedan anotadas aqui por si se decide sumarlas.</t>
         </is>
       </c>
       <c r="J46" s="2" t="n"/>

</xml_diff>

<commit_message>
control de subida de videos de la bodycam
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -17208,7 +17208,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>BC-7, BC-8, BC-9, BC-10, BC-11</t>
+          <t>BC-7, BC-8, BC-9, BC-10, BC-11, BC-12, BC-13</t>
         </is>
       </c>
       <c r="L5" s="13">
@@ -17216,7 +17216,7 @@
         <v/>
       </c>
       <c r="M5" s="13" t="n">
-        <v>3972</v>
+        <v>4637</v>
       </c>
       <c r="N5" s="13">
         <f>SUMIFS($D$4:$D$55,$B$4:$B$55,"BC",$G$4:$G$55,"&lt;&gt;Sí")</f>
@@ -17271,7 +17271,7 @@
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>AN-2, AN-3, AN-4, AN-5, AN-6, AN-7, AN-8, AN-9, AN-10, AN-11</t>
+          <t>AN-2, AN-3, AN-4, AN-5, AN-6, AN-7, AN-8, AN-9, AN-10, AN-11, AN-12</t>
         </is>
       </c>
       <c r="L6" s="13">
@@ -17279,7 +17279,7 @@
         <v/>
       </c>
       <c r="M6" s="13" t="n">
-        <v>18696</v>
+        <v>19128</v>
       </c>
       <c r="N6" s="13">
         <f>SUMIFS($D$4:$D$55,$B$4:$B$55,"AN",$G$4:$G$55,"&lt;&gt;Sí")</f>
@@ -19143,14 +19143,42 @@
       <c r="O48" s="2" t="n"/>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="15">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="11" t="n"/>
-      <c r="C49" s="11" t="n"/>
-      <c r="D49" s="11" t="n"/>
-      <c r="E49" s="11" t="n"/>
-      <c r="F49" s="11" t="n"/>
-      <c r="G49" s="11" t="n"/>
-      <c r="H49" s="11" t="n"/>
+      <c r="A49" s="6" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>BC-12</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>Modo kiosco de la unidad (device owner), rama dev_device_owner. La app pasa a ser propietaria del aparato: anclaje de pantalla solo para nuestro paquete, barra de estado desactivada, la app como lanzador, apps del fabricante escondidas y restricciones (sin reset de fabrica, sin modo seguro, sin cambiar la hora). Dos reglas fijas: adb NUNCA se corta (las politicas fuerzan ADB_ENABLED y se deja fuera DISALLOW_INSTALL_APPS, que bloquearia adb install) y siempre hay salida sin borrar (clearDeviceOwnerApp). De regalo: arranque automatico real siendo lanzador, setTime para las 6 h de desfase y permisos concedidos solos. Script tools/kiosco.sh con dos niveles, piloto (sin rol, reversible, recorre todas las unidades conectadas) y kiosco completo. Incluye el analisis de las tres vias posibles (kiosco, firmware a medida y ROM propia sobre AOSP) y el destripado de la APK del fabricante MCP_..._ZXA_v286 (com.smarteye.mcu): resulto ser una app de usuario firmada con clave de depuracion, lanzador mas device admin, sin lock task ni nada del rol de propietario. COMPILA, SIN PROBAR EN LA UNIDAD: no habia aparato conectado</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>indicado por el usuario: 3 h para el dia; reparto por app y tarea estimado sobre ese total</t>
+        </is>
+      </c>
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="n"/>
@@ -19159,14 +19187,42 @@
       <c r="O49" s="2" t="n"/>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="15">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="11" t="n"/>
-      <c r="C50" s="11" t="n"/>
-      <c r="D50" s="11" t="n"/>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="11" t="n"/>
-      <c r="H50" s="11" t="n"/>
+      <c r="A50" s="6" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>BC-13</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>Cancelar la subida de un incidente, lado bodycam. Diagnostico de por que INC_000032 se subia una y otra vez: resumePending reencola en cada arranque y en cada apertura de la app todo incidente sin recibo de entrega, y el reintento no se rinde nunca por diseno. UploadCancel marca el incidente con un fichero dentro de su propio directorio (sobrevive a reinstalar y viaja con el incidente), ChunkedUploader corta ENTRE bloques (nunca a mitad de un PATCH) y mira la cancelacion en rodajas de 500 ms durante la espera entre reintentos. Cancelar NO borra el video: lo saca de la cola y se puede reencolar sin repetir un byte. Comandos BT UPLOAD_LIST, UPLOAD_CANCEL y UPLOAD_RESUME, mas atajo por adb. COMPILA, SIN PROBAR EN LA UNIDAD</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>indicado por el usuario: 3 h para el dia; reparto por app y tarea estimado sobre ese total</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="n"/>
       <c r="K50" s="2" t="n"/>
       <c r="L50" s="2" t="n"/>
@@ -19175,14 +19231,42 @@
       <c r="O50" s="2" t="n"/>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="15">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="11" t="n"/>
-      <c r="C51" s="11" t="n"/>
-      <c r="D51" s="11" t="n"/>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="11" t="n"/>
-      <c r="H51" s="11" t="n"/>
+      <c r="A51" s="6" t="n">
+        <v>46285</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>AN-12</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>Pantalla de subidas de la bodycam en el movil. El telefono es el unico sitio con pantalla para ver la lista y decidir: la de la unidad mide 3 cm. Modelo SubidaDeEvidencia y flujo subidas en BodycamRepository (la lista llega en la linea UPLOADS y NO viaja en el STATUS de cada 5 s, que puede tener decenas de incidentes y no cambia sola), pantalla con tres estados DELIVERED / PENDING / CANCELLED, boton CANCEL con dialogo de confirmacion y QUEUE AGAIN para devolver a la cola, y ruta bodycam/uploads con boton UPLOADS en el controlador. El dialogo dice expresamente que el video se queda en la camara: si diera a entender que borra, nadie lo usaria. COMPILA, SIN PROBAR CON APARATOS</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>indicado por el usuario: 3 h para el dia; reparto por app y tarea estimado sobre ese total</t>
+        </is>
+      </c>
       <c r="J51" s="2" t="n"/>
       <c r="K51" s="2" t="n"/>
       <c r="L51" s="2" t="n"/>
@@ -19296,7 +19380,7 @@
     <row r="58" ht="57.75" customHeight="1" s="15">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.   15 DE SEPTIEMBRE: AN-4 y BC-8 (PTT). BC-8 = la bodycam escucha el canal todo el tiempo para que el PTT de los telefonos suene por su altavoz (punto 1 de los requisitos del 14-sep). AN-4 = boton de PTT del telefono de un toque, y diagnostico de que Nexus no vuelve al canal tras perder la conexion (documentado, sin arreglar). Las horas salen del reloj de sesion 12:28-13:07 (0,65 h medidas), redondeadas al alza a 1 h; el reparto 0,5 / 0,5 es estimacion sobre las marcas de fichero (BodyCamServer 12:34-12:49, Nexus 12:59-13:04). Lineas del 15, sin commitear, medidas con git: 308 anadidas en BC (de ellas 279 en LivestreamService, reescrito: salen tambien 216) y 22 en AN.   15 DE SEPTIEMBRE, TARDE: AN-4 = reconexion al canal de Agora (el telefono se quedaba fuera sin avisar). AN-2 = revision del IAM y workflows 5 (cambio de PIN) y 30 (fin de turno). AN-10 (bloque nuevo) = auditoria local, workflows 61 y 46. Las horas salen del reloj de sesion 13:34-14:05 y 14:22-15:06 (1,25 h medidas), redondeadas al alza a 1,5 h; el reparto 0,3 / 0,6 / 0,6 es estimacion sobre la hora de cada peticion. NO se cuentan 13:20-13:34, que fue anotar en esta tabla las horas de la manana, ni 14:05-14:22, espera a que se desbloqueara el telefono de pruebas. Lineas .kt: 176 de la reconexion (commit 49d8c20, sin las 22 del boton de PTT ya contadas en la fila 33); unas 529 de los wf 5 y 30 y unas 903 de los wf 61 y 46, de ellas 96 de pruebas JVM, sin commitear; el reparto entre bloques de los ficheros compartidos (IdentityRepository, ProfileScreen, AppNavHost, AppContainer) es estimacion.   15 DE SEPTIEMBRE, FINAL DE LA TARDE: AN-5 (gafas) = selector de gafas sin MAC compilada, y arreglo de la conexion en Android 11 (el SDK del fabricante comprobaba un permiso que en esa version no existe). Las 2 h las indico el usuario; la sesion registra 0,85 h activas (15:06-15:27, 16:03-16:26 y 16:41-16:48) y los huecos 15:27-16:03 y 16:26-16:41 fueron del usuario con la release del manager y las pruebas en el Redmi. Reparto 1 / 1 estimado. Lineas .kt sin commitear, medidas con git: 378 (unas 343 del selector y unas 35 del arreglo de Android 11).   15 DE SEPTIEMBRE, NOCHE: AN-4 (PTT) = aviso de PTT pisado, con tono de tres pitidos y boton ambar cuando dos agentes hablan a la vez. La hora la indico el usuario. Lineas .kt sin commitear, medidas con git: 126 en AN (19 del atajo de debug) y 11 en BC (el tono gemelo en PttTones).   RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33 y el 15-sep a la 43; el total esta en la fila 44 y esta leyenda en la 46. El 18-sep se amplio a la 55: total en la 56 y esta leyenda en la 58. Libres las filas 49-55. Al volver a ampliar, cambiar $55 en D56 y en K8, L5-L8 y N5-N7.   16 Y 17 DE SEPTIEMBRE, BACKEND (aplicacion NX, nueva): NX es el tercer repositorio, aeria-nexus, que hasta hoy no estaba en este libro aunque llevaba dos dias de trabajo. Django 5 + DRF + Celery y el panel Next.js, mas el repositorio de contratos aeria-contracts, que se imputa aqui porque nacio dentro de estas mismas sesiones. NX-1 = contratos, simulador de cliente, costuras de portabilidad e identidad F1-F6. NX-2 = ingesta de evidencia por tus y enlace de la subida con el analisis. NX-3 = coste medido, arreglos y puesta a punto para la demostracion al manager.   ORIGEN DE LAS HORAS DEL BACKEND: las dos filas del 16 salen de las marcas de los commits, 15:32 (primer commit de contratos) a 23:42 (ultimo del backend), 8,15 h medidas; el corte entre NX-1 y NX-2 es el commit de las 18:47, que cierra identidad. Cada tramo se redondea al alza al medio punto por separado (3,25-&gt;3,5 y 4,9-&gt;5), asi que la suma imputada del dia es 8,5. NO se cuenta nada anterior al primer commit. Las 2,5 h del 17 las indico el usuario: esa sesion no dejo commits, se prolongo pasada la medianoche y se imputa entera al 17.   LINEAS DE CODIGO DEL BACKEND: 10.475, medidas con git y contando solo codigo (.py, .ts, .tsx). Del 16 son 9.871 en diez commits; del 17, 604 sin commitear (469 de cuatro ficheros nuevos y 135 de modificaciones). NO se cuentan 2.210 lineas de documentacion en Markdown de los dos dias, ni las 1.028 del simulador de cliente y 456 del OpenAPI que viven en aeria-contracts, aunque se escribieran en estas sesiones: quedan anotadas aqui por si se decide sumarlas.   18 DE SEPTIEMBRE: NX-4 (bloque nuevo) = evidencia del telefono en el backend y el panel. AN-11 (bloque nuevo) = conexion de la app con el backend (IAM real, sesion, subida autenticada, manifiesto y ubicacion). NX-1 y NX-3 se reutilizan para el acceso al panel y los arreglos del panel de la manana.   ORIGEN DE LAS HORAS DEL 18: el total de 4 h lo indico el usuario. El reloj de la sesion de backend va de 10:15:48 a 14:28:12 (4,21 h) y la sesion de la app siguio hasta las 15:25; las marcas de fichero (10:58, 11:23, 12:27, 13:40) lo corroboran. El reparto 0,8 / 0,4 / 1,3 / 1,5 entre los tramos A, B y C (backend y app) es estimacion sobre ese total.   LINEAS DEL 18, sin commitear: NX 833 medidas con git sin documentacion (tramo A +209, B +105 y C +519); AN 933 (511 en ficheros existentes y 422 en nuevos). NO se cuentan las 121 lineas de documentacion de aeria-contracts.   18 DE SEPTIEMBRE, BODYCAM: BC-11 (bloque nuevo) = modo noche automatico de la W1 (LEDs IR, filtro IR-CUT, sensor de luz y blanco y negro en grabacion y SOS). Las horas salen de las marcas de fichero y del reloj de sesion 15:21-16:42 (1,35 h medidas), redondeadas al alza a 1,5 h; incluyen las dos pruebas en la unidad. Lineas .kt sin commitear, medidas con git: 310 en BC (253 en ModoNoche y MonocromoSos, nuevos, y 57 en modificaciones). El SOS en monocromo compila y esta instalado, pero queda pendiente de probar con la unidad.</t>
+          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.   15 DE SEPTIEMBRE: AN-4 y BC-8 (PTT). BC-8 = la bodycam escucha el canal todo el tiempo para que el PTT de los telefonos suene por su altavoz (punto 1 de los requisitos del 14-sep). AN-4 = boton de PTT del telefono de un toque, y diagnostico de que Nexus no vuelve al canal tras perder la conexion (documentado, sin arreglar). Las horas salen del reloj de sesion 12:28-13:07 (0,65 h medidas), redondeadas al alza a 1 h; el reparto 0,5 / 0,5 es estimacion sobre las marcas de fichero (BodyCamServer 12:34-12:49, Nexus 12:59-13:04). Lineas del 15, sin commitear, medidas con git: 308 anadidas en BC (de ellas 279 en LivestreamService, reescrito: salen tambien 216) y 22 en AN.   15 DE SEPTIEMBRE, TARDE: AN-4 = reconexion al canal de Agora (el telefono se quedaba fuera sin avisar). AN-2 = revision del IAM y workflows 5 (cambio de PIN) y 30 (fin de turno). AN-10 (bloque nuevo) = auditoria local, workflows 61 y 46. Las horas salen del reloj de sesion 13:34-14:05 y 14:22-15:06 (1,25 h medidas), redondeadas al alza a 1,5 h; el reparto 0,3 / 0,6 / 0,6 es estimacion sobre la hora de cada peticion. NO se cuentan 13:20-13:34, que fue anotar en esta tabla las horas de la manana, ni 14:05-14:22, espera a que se desbloqueara el telefono de pruebas. Lineas .kt: 176 de la reconexion (commit 49d8c20, sin las 22 del boton de PTT ya contadas en la fila 33); unas 529 de los wf 5 y 30 y unas 903 de los wf 61 y 46, de ellas 96 de pruebas JVM, sin commitear; el reparto entre bloques de los ficheros compartidos (IdentityRepository, ProfileScreen, AppNavHost, AppContainer) es estimacion.   15 DE SEPTIEMBRE, FINAL DE LA TARDE: AN-5 (gafas) = selector de gafas sin MAC compilada, y arreglo de la conexion en Android 11 (el SDK del fabricante comprobaba un permiso que en esa version no existe). Las 2 h las indico el usuario; la sesion registra 0,85 h activas (15:06-15:27, 16:03-16:26 y 16:41-16:48) y los huecos 15:27-16:03 y 16:26-16:41 fueron del usuario con la release del manager y las pruebas en el Redmi. Reparto 1 / 1 estimado. Lineas .kt sin commitear, medidas con git: 378 (unas 343 del selector y unas 35 del arreglo de Android 11).   15 DE SEPTIEMBRE, NOCHE: AN-4 (PTT) = aviso de PTT pisado, con tono de tres pitidos y boton ambar cuando dos agentes hablan a la vez. La hora la indico el usuario. Lineas .kt sin commitear, medidas con git: 126 en AN (19 del atajo de debug) y 11 en BC (el tono gemelo en PttTones).   RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33 y el 15-sep a la 43; el total esta en la fila 44 y esta leyenda en la 46. El 18-sep se amplio a la 55: total en la 56 y esta leyenda en la 58. Libres las filas 49-55. Al volver a ampliar, cambiar $55 en D56 y en K8, L5-L8 y N5-N7.   16 Y 17 DE SEPTIEMBRE, BACKEND (aplicacion NX, nueva): NX es el tercer repositorio, aeria-nexus, que hasta hoy no estaba en este libro aunque llevaba dos dias de trabajo. Django 5 + DRF + Celery y el panel Next.js, mas el repositorio de contratos aeria-contracts, que se imputa aqui porque nacio dentro de estas mismas sesiones. NX-1 = contratos, simulador de cliente, costuras de portabilidad e identidad F1-F6. NX-2 = ingesta de evidencia por tus y enlace de la subida con el analisis. NX-3 = coste medido, arreglos y puesta a punto para la demostracion al manager.   ORIGEN DE LAS HORAS DEL BACKEND: las dos filas del 16 salen de las marcas de los commits, 15:32 (primer commit de contratos) a 23:42 (ultimo del backend), 8,15 h medidas; el corte entre NX-1 y NX-2 es el commit de las 18:47, que cierra identidad. Cada tramo se redondea al alza al medio punto por separado (3,25-&gt;3,5 y 4,9-&gt;5), asi que la suma imputada del dia es 8,5. NO se cuenta nada anterior al primer commit. Las 2,5 h del 17 las indico el usuario: esa sesion no dejo commits, se prolongo pasada la medianoche y se imputa entera al 17.   LINEAS DE CODIGO DEL BACKEND: 10.475, medidas con git y contando solo codigo (.py, .ts, .tsx). Del 16 son 9.871 en diez commits; del 17, 604 sin commitear (469 de cuatro ficheros nuevos y 135 de modificaciones). NO se cuentan 2.210 lineas de documentacion en Markdown de los dos dias, ni las 1.028 del simulador de cliente y 456 del OpenAPI que viven en aeria-contracts, aunque se escribieran en estas sesiones: quedan anotadas aqui por si se decide sumarlas.   18 DE SEPTIEMBRE: NX-4 (bloque nuevo) = evidencia del telefono en el backend y el panel. AN-11 (bloque nuevo) = conexion de la app con el backend (IAM real, sesion, subida autenticada, manifiesto y ubicacion). NX-1 y NX-3 se reutilizan para el acceso al panel y los arreglos del panel de la manana.   ORIGEN DE LAS HORAS DEL 18: el total de 4 h lo indico el usuario. El reloj de la sesion de backend va de 10:15:48 a 14:28:12 (4,21 h) y la sesion de la app siguio hasta las 15:25; las marcas de fichero (10:58, 11:23, 12:27, 13:40) lo corroboran. El reparto 0,8 / 0,4 / 1,3 / 1,5 entre los tramos A, B y C (backend y app) es estimacion sobre ese total.   LINEAS DEL 18, sin commitear: NX 833 medidas con git sin documentacion (tramo A +209, B +105 y C +519); AN 933 (511 en ficheros existentes y 422 en nuevos). NO se cuentan las 121 lineas de documentacion de aeria-contracts.   18 DE SEPTIEMBRE, BODYCAM: BC-11 (bloque nuevo) = modo noche automatico de la W1 (LEDs IR, filtro IR-CUT, sensor de luz y blanco y negro en grabacion y SOS). Las horas salen de las marcas de fichero y del reloj de sesion 15:21-16:42 (1,35 h medidas), redondeadas al alza a 1,5 h; incluyen las dos pruebas en la unidad. Lineas .kt sin commitear, medidas con git: 310 en BC (253 en ModoNoche y MonocromoSos, nuevos, y 57 en modificaciones). El SOS en monocromo compila y esta instalado, pero queda pendiente de probar con la unidad.   20 DE SEPTIEMBRE: BC-12 (bloque nuevo) = modo kiosco de la unidad con device owner, en la rama dev_device_owner, mas el analisis de las tres vias de control y el destripado de la APK del fabricante. BC-13 y AN-12 (bloques nuevos) = cancelar desde el movil la subida de un incidente, que hasta hoy no se podia parar nunca. Las 3 h del dia las indico el usuario; el reparto 1,5 / 0,5 / 1 es estimacion. NADA de lo de hoy se ha probado en aparatos: no habia ni bodycam ni telefono conectados, las dos apps solo compilan. Lineas .kt sin commitear, medidas con git: 665 en BC (535 de tres ficheros nuevos, DeviceOwner, FalconDeviceAdmin y UploadCancel, y 130 de modificaciones) y 432 en AN (353 de dos ficheros nuevos y 79 de modificaciones); el reparto de las lineas de BC entre BC-12 y BC-13 es estimacion. NO se cuentan las lineas de tools/kiosco.sh ni las de los dos DEVLOG.   FILAS LIBRES: quedan 52-55; al agotarlas hay que ampliar $55 en D56, K8, L5-L8 y N5-N7.</t>
         </is>
       </c>
       <c r="J58" s="2" t="n"/>

</xml_diff>

<commit_message>
sos con directo desde el mapa, silencios y tono configurable, el movil suelta la bodycam al cerrar sesion y caducidad de la credencial
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -17220,7 +17220,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>BC-7, BC-8, BC-9, BC-10, BC-11, BC-12, BC-13, BC-14</t>
+          <t>BC-7, BC-8, BC-9, BC-10, BC-11, BC-12, BC-13, BC-14, BC-16</t>
         </is>
       </c>
       <c r="L5" s="13">
@@ -17228,7 +17228,7 @@
         <v/>
       </c>
       <c r="M5" s="13" t="n">
-        <v>5466</v>
+        <v>5560</v>
       </c>
       <c r="N5" s="13">
         <f>SUMIFS($D$4:$D$65,$B$4:$B$65,"BC",$G$4:$G$65,"&lt;&gt;Sí")</f>
@@ -17283,7 +17283,7 @@
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>AN-2, AN-3, AN-4, AN-5, AN-6, AN-7, AN-8, AN-9, AN-10, AN-11, AN-12</t>
+          <t>AN-2, AN-3, AN-4, AN-5, AN-6, AN-7, AN-8, AN-9, AN-10, AN-11, AN-12, AN-13</t>
         </is>
       </c>
       <c r="L6" s="13">
@@ -17291,7 +17291,7 @@
         <v/>
       </c>
       <c r="M6" s="13" t="n">
-        <v>19554</v>
+        <v>20950</v>
       </c>
       <c r="N6" s="13">
         <f>SUMIFS($D$4:$D$65,$B$4:$B$65,"AN",$G$4:$G$65,"&lt;&gt;Sí")</f>
@@ -19495,14 +19495,42 @@
       <c r="O56" s="2" t="n"/>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="15">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="11" t="n"/>
-      <c r="C57" s="11" t="n"/>
-      <c r="D57" s="11" t="n"/>
-      <c r="E57" s="11" t="n"/>
-      <c r="F57" s="11" t="n"/>
-      <c r="G57" s="11" t="n"/>
-      <c r="H57" s="11" t="n"/>
+      <c r="A57" s="6" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>BC-7</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E57" s="11" t="inlineStr">
+        <is>
+          <t>Identidad de la bodycam y alta en el IAM (opcion B). El BWC-xxxx pasa a salir del serial (4 hex del SHA-256 de Build.getSerial()): reinstalar ya no cambia el id ni deja huerfana la credencial; el choque entre unidades lo para el guion antes de mandar nada. READ_PHONE_STATE concedido por el device owner o por el guion. Alta de la W1 contra el backend: BWC-7D6F, certificado de AeriaOne Device Identity CA y las dos anclas, PROBADO EN LA UNIDAD. Analisis de contestar al SOS por voz (PTT en el directo), encargado a la sesion AN</t>
+        </is>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>58493ba + sin commitear</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H57" s="11" t="inlineStr">
+        <is>
+          <t>reloj de sesion 23:25-23:58 (0,55 h), redondeado al alza; la sesion entera 23:25-00:20 se parte en dos filas</t>
+        </is>
+      </c>
       <c r="J57" s="2" t="n"/>
       <c r="K57" s="2" t="n"/>
       <c r="L57" s="2" t="n"/>
@@ -19511,14 +19539,42 @@
       <c r="O57" s="2" t="n"/>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="15">
-      <c r="A58" s="6" t="n"/>
-      <c r="B58" s="11" t="n"/>
-      <c r="C58" s="11" t="n"/>
-      <c r="D58" s="11" t="n"/>
-      <c r="E58" s="11" t="n"/>
-      <c r="F58" s="11" t="n"/>
-      <c r="G58" s="11" t="n"/>
-      <c r="H58" s="11" t="n"/>
+      <c r="A58" s="6" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>BC-16</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>Alta de aparatos a distancia para el manager, que prueba en otro pais sin ordenador y con APK de release: analisis de por que no se conectan (el alta solo va por adb), propuesta de alta de la bodycam a traves del movil para el 29-sep y version piloto sin identidad (flag PILOTO_SIN_IDENTIDAD en la bodycam; el movil ya lo cubre con SIMULADOR_CONFIANZA_EN_RELEASE). COMPILA A MEDIAS: la compilacion final quedo bloqueada por permisos</t>
+        </is>
+      </c>
+      <c r="F58" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G58" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="inlineStr">
+        <is>
+          <t>reloj de sesion 23:58-00:20 (0,4 h), redondeado al alza</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="n"/>
       <c r="K58" s="2" t="n"/>
       <c r="L58" s="2" t="n"/>
@@ -19527,14 +19583,42 @@
       <c r="O58" s="2" t="n"/>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="15">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="11" t="n"/>
-      <c r="C59" s="11" t="n"/>
-      <c r="D59" s="11" t="n"/>
-      <c r="E59" s="11" t="n"/>
-      <c r="F59" s="11" t="n"/>
-      <c r="G59" s="11" t="n"/>
-      <c r="H59" s="11" t="n"/>
+      <c r="A59" s="6" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>AN-2</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>AN-0: el telefono guarda el ancla de perifericos (device_ca_pem) que le devuelve su propia alta, sin la cual rechazaria a una W1 dada de alta en el IAM. Wf 53: con la credencial caducada el telefono se bloquea salvo mientras graba (camara, audio, SOS, bodycam o gafas), y desata la W1 con el motivo CADUCIDAD. Compila y pasan las pruebas de la politica; SIN PROBAR EN APARATO</t>
+        </is>
+      </c>
+      <c r="F59" s="11" t="inlineStr">
+        <is>
+          <t>2516769 + sin commitear</t>
+        </is>
+      </c>
+      <c r="G59" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H59" s="11" t="inlineStr">
+        <is>
+          <t>marcas de fichero de la sesion AN: 23:20-23:30 y 23:40-23:55; los 35 min de la sesion AN se redondean al alza a 1 h y se reparten 0,5 / 0,5</t>
+        </is>
+      </c>
       <c r="J59" s="2" t="n"/>
       <c r="K59" s="2" t="n"/>
       <c r="L59" s="2" t="n"/>
@@ -19543,14 +19627,42 @@
       <c r="O59" s="2" t="n"/>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="15">
-      <c r="A60" s="6" t="n"/>
-      <c r="B60" s="11" t="n"/>
-      <c r="C60" s="11" t="n"/>
-      <c r="D60" s="11" t="n"/>
-      <c r="E60" s="11" t="n"/>
-      <c r="F60" s="11" t="n"/>
-      <c r="G60" s="11" t="n"/>
-      <c r="H60" s="11" t="n"/>
+      <c r="A60" s="6" t="n">
+        <v>46293</v>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>AN-4</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>PTT en el directo del SOS: boton de mantener para hablar en la pantalla del livestream, para que los agentes que ven un SOS puedan contestar al que lo emite (decision del usuario: voz por PTT, ni texto ni conferencia). Mismos tonos y permiso que en Operations, aviso de PTT pisado; la banda de quien habla baja para no tapar el boton de volver. Compila, SIN PROBAR EN APARATO</t>
+        </is>
+      </c>
+      <c r="F60" s="11" t="inlineStr">
+        <is>
+          <t>2516769</t>
+        </is>
+      </c>
+      <c r="G60" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H60" s="11" t="inlineStr">
+        <is>
+          <t>marcas de fichero de la sesion AN: 23:30-23:40; ver fila anterior para el redondeo</t>
+        </is>
+      </c>
       <c r="J60" s="2" t="n"/>
       <c r="K60" s="2" t="n"/>
       <c r="L60" s="2" t="n"/>
@@ -19559,14 +19671,42 @@
       <c r="O60" s="2" t="n"/>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="15">
-      <c r="A61" s="6" t="n"/>
-      <c r="B61" s="11" t="n"/>
-      <c r="C61" s="11" t="n"/>
-      <c r="D61" s="11" t="n"/>
-      <c r="E61" s="11" t="n"/>
-      <c r="F61" s="11" t="n"/>
-      <c r="G61" s="11" t="n"/>
-      <c r="H61" s="11" t="n"/>
+      <c r="A61" s="6" t="n">
+        <v>46294</v>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>AN-13</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>SOS con directo (peticion del usuario). Mapa: el circulo amarillo de un agente en SOS se puede tocar y abre el aviso SOS active / VIEW LIVESTREAM (dos botones si emite desde el telefono y la bodycam); el telefono atado anuncia su bodycam en la posicion para situar en el mapa el SOS de la W1, que no tiene GPS. Directo del receptor: PTT conmutador (boton sacado de Operations a ui/components) y MUTED local. Directo del emisor: MIC ON/OFF (arranca abierto) y OTHERS ON/OFF, solo volumen local para no perder nada en la grabacion de la nube, con registro en el diario de auditoria. Tono de SOS configurable (OFF / DISCREET / LOUD) en el perfil, mandado a la W1 por BT (SOS_TONE); camara y micro se publican al acabar el tono. Coordinacion con la sesion de la bodycam (doble F2 en lugar de pulsacion larga, que el firmware no permite; micro abierto en el SOS de la W1). Probado en el Samsung y la W1: SOS_TONE, tono, micro y silencios, restauracion al cancelar, diario y directo de la W1 con MUTED. Arreglados en la prueba: banda de PTT que tapaba la barra del directo y texto partido.</t>
+        </is>
+      </c>
+      <c r="F61" s="11" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G61" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H61" s="11" t="inlineStr">
+        <is>
+          <t>indicado por el usuario: 2,5 h. Reloj de la sesion: ~13:10-13:55 y 14:58-15:10 (~0,95 h medidas, inicio estimado); el resto es el tiempo del usuario instalando y probando a mano</t>
+        </is>
+      </c>
       <c r="J61" s="2" t="n"/>
       <c r="K61" s="2" t="n"/>
       <c r="L61" s="2" t="n"/>
@@ -19680,7 +19820,7 @@
     <row r="68" ht="57.75" customHeight="1" s="15">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.   15 DE SEPTIEMBRE: AN-4 y BC-8 (PTT). BC-8 = la bodycam escucha el canal todo el tiempo para que el PTT de los telefonos suene por su altavoz (punto 1 de los requisitos del 14-sep). AN-4 = boton de PTT del telefono de un toque, y diagnostico de que Nexus no vuelve al canal tras perder la conexion (documentado, sin arreglar). Las horas salen del reloj de sesion 12:28-13:07 (0,65 h medidas), redondeadas al alza a 1 h; el reparto 0,5 / 0,5 es estimacion sobre las marcas de fichero (BodyCamServer 12:34-12:49, Nexus 12:59-13:04). Lineas del 15, sin commitear, medidas con git: 308 anadidas en BC (de ellas 279 en LivestreamService, reescrito: salen tambien 216) y 22 en AN.   15 DE SEPTIEMBRE, TARDE: AN-4 = reconexion al canal de Agora (el telefono se quedaba fuera sin avisar). AN-2 = revision del IAM y workflows 5 (cambio de PIN) y 30 (fin de turno). AN-10 (bloque nuevo) = auditoria local, workflows 61 y 46. Las horas salen del reloj de sesion 13:34-14:05 y 14:22-15:06 (1,25 h medidas), redondeadas al alza a 1,5 h; el reparto 0,3 / 0,6 / 0,6 es estimacion sobre la hora de cada peticion. NO se cuentan 13:20-13:34, que fue anotar en esta tabla las horas de la manana, ni 14:05-14:22, espera a que se desbloqueara el telefono de pruebas. Lineas .kt: 176 de la reconexion (commit 49d8c20, sin las 22 del boton de PTT ya contadas en la fila 33); unas 529 de los wf 5 y 30 y unas 903 de los wf 61 y 46, de ellas 96 de pruebas JVM, sin commitear; el reparto entre bloques de los ficheros compartidos (IdentityRepository, ProfileScreen, AppNavHost, AppContainer) es estimacion.   15 DE SEPTIEMBRE, FINAL DE LA TARDE: AN-5 (gafas) = selector de gafas sin MAC compilada, y arreglo de la conexion en Android 11 (el SDK del fabricante comprobaba un permiso que en esa version no existe). Las 2 h las indico el usuario; la sesion registra 0,85 h activas (15:06-15:27, 16:03-16:26 y 16:41-16:48) y los huecos 15:27-16:03 y 16:26-16:41 fueron del usuario con la release del manager y las pruebas en el Redmi. Reparto 1 / 1 estimado. Lineas .kt sin commitear, medidas con git: 378 (unas 343 del selector y unas 35 del arreglo de Android 11).   15 DE SEPTIEMBRE, NOCHE: AN-4 (PTT) = aviso de PTT pisado, con tono de tres pitidos y boton ambar cuando dos agentes hablan a la vez. La hora la indico el usuario. Lineas .kt sin commitear, medidas con git: 126 en AN (19 del atajo de debug) y 11 en BC (el tono gemelo en PttTones).   RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33 y el 15-sep a la 43; el total esta en la fila 44 y esta leyenda en la 46. El 18-sep se amplio a la 55: total en la 56 y esta leyenda en la 58. Libres las filas 49-55. Al volver a ampliar, cambiar $55 en D56 y en K8, L5-L8 y N5-N7.   16 Y 17 DE SEPTIEMBRE, BACKEND (aplicacion NX, nueva): NX es el tercer repositorio, aeria-nexus, que hasta hoy no estaba en este libro aunque llevaba dos dias de trabajo. Django 5 + DRF + Celery y el panel Next.js, mas el repositorio de contratos aeria-contracts, que se imputa aqui porque nacio dentro de estas mismas sesiones. NX-1 = contratos, simulador de cliente, costuras de portabilidad e identidad F1-F6. NX-2 = ingesta de evidencia por tus y enlace de la subida con el analisis. NX-3 = coste medido, arreglos y puesta a punto para la demostracion al manager.   ORIGEN DE LAS HORAS DEL BACKEND: las dos filas del 16 salen de las marcas de los commits, 15:32 (primer commit de contratos) a 23:42 (ultimo del backend), 8,15 h medidas; el corte entre NX-1 y NX-2 es el commit de las 18:47, que cierra identidad. Cada tramo se redondea al alza al medio punto por separado (3,25-&gt;3,5 y 4,9-&gt;5), asi que la suma imputada del dia es 8,5. NO se cuenta nada anterior al primer commit. Las 2,5 h del 17 las indico el usuario: esa sesion no dejo commits, se prolongo pasada la medianoche y se imputa entera al 17.   LINEAS DE CODIGO DEL BACKEND: 10.475, medidas con git y contando solo codigo (.py, .ts, .tsx). Del 16 son 9.871 en diez commits; del 17, 604 sin commitear (469 de cuatro ficheros nuevos y 135 de modificaciones). NO se cuentan 2.210 lineas de documentacion en Markdown de los dos dias, ni las 1.028 del simulador de cliente y 456 del OpenAPI que viven en aeria-contracts, aunque se escribieran en estas sesiones: quedan anotadas aqui por si se decide sumarlas.   18 DE SEPTIEMBRE: NX-4 (bloque nuevo) = evidencia del telefono en el backend y el panel. AN-11 (bloque nuevo) = conexion de la app con el backend (IAM real, sesion, subida autenticada, manifiesto y ubicacion). NX-1 y NX-3 se reutilizan para el acceso al panel y los arreglos del panel de la manana.   ORIGEN DE LAS HORAS DEL 18: el total de 4 h lo indico el usuario. El reloj de la sesion de backend va de 10:15:48 a 14:28:12 (4,21 h) y la sesion de la app siguio hasta las 15:25; las marcas de fichero (10:58, 11:23, 12:27, 13:40) lo corroboran. El reparto 0,8 / 0,4 / 1,3 / 1,5 entre los tramos A, B y C (backend y app) es estimacion sobre ese total.   LINEAS DEL 18, sin commitear: NX 833 medidas con git sin documentacion (tramo A +209, B +105 y C +519); AN 933 (511 en ficheros existentes y 422 en nuevos). NO se cuentan las 121 lineas de documentacion de aeria-contracts.   18 DE SEPTIEMBRE, BODYCAM: BC-11 (bloque nuevo) = modo noche automatico de la W1 (LEDs IR, filtro IR-CUT, sensor de luz y blanco y negro en grabacion y SOS). Las horas salen de las marcas de fichero y del reloj de sesion 15:21-16:42 (1,35 h medidas), redondeadas al alza a 1,5 h; incluyen las dos pruebas en la unidad. Lineas .kt sin commitear, medidas con git: 310 en BC (253 en ModoNoche y MonocromoSos, nuevos, y 57 en modificaciones). El SOS en monocromo compila y esta instalado, pero queda pendiente de probar con la unidad.   20 DE SEPTIEMBRE: BC-12 (bloque nuevo) = modo kiosco de la unidad con device owner, en la rama dev_device_owner, mas el analisis de las tres vias de control y el destripado de la APK del fabricante. BC-13 y AN-12 (bloques nuevos) = cancelar desde el movil la subida de un incidente, que hasta hoy no se podia parar nunca. Las 3 h del dia las indico el usuario; el reparto 1,5 / 0,5 / 1 es estimacion. NADA de lo de hoy se ha probado en aparatos: no habia ni bodycam ni telefono conectados, las dos apps solo compilan. Lineas .kt sin commitear, medidas con git: 665 en BC (535 de tres ficheros nuevos, DeviceOwner, FalconDeviceAdmin y UploadCancel, y 130 de modificaciones) y 432 en AN (353 de dos ficheros nuevos y 79 de modificaciones); el reparto de las lineas de BC entre BC-12 y BC-13 es estimacion. NO se cuentan las lineas de tools/kiosco.sh ni las de los dos DEVLOG.   21 DE SEPTIEMBRE: BC-11 (modo noche, ya existente) = arreglo de los LEDs infrarrojos, que no se apagaban al parar de grabar, del giro de la pantalla de MainActivity y, en la sesion de la noche, del apagado de la unidad, que dejaba los infrarrojos encendidos con la bodycam apagada. Los tres fallos los observo el usuario en la unidad. Va en BC-11 y no en un bloque nuevo porque todo es corregir el modo noche entregado el 18-sep. DECISION DEL USUARIO: los IR se apagan al parar la grabacion, aunque el anillo siga armado; queda por validar con el cliente que el pre-roll nocturno de 20 s se grabe sin ellos. HORAS: las indico el usuario, que fijo la imputacion el 21-sep a las 21:00 y las subio de 1 a 1,5 h al cerrar la sesion de la noche; el trabajo se hizo entre la tarde del 20-sep y la madrugada del 21. PROBADO EN LA UNIDAD, a diferencia de lo que decia esta leyenda antes: con la bodycam por adb se midio el apagado (infrarrojo encendido 1441 lux, apagado 0) y el usuario confirmo el apagado real desde el boton. El ensayo hizo falta montarlo aparte porque ACTION_SHUTDOWN es un broadcast protegido que adb no puede enviar y la unidad es build user sin root. Medido de paso: la escritura del motor del filtro IR-CUT bloquea 2070 ms, frente a 27-44 ms de cada luz. Lineas .kt sin commitear, medidas con git: 107 anadidas y 20 borradas de la primera sesion, mas unas 230 anadidas (112 de ellas ApagadoReceiver, fichero nuevo) y 21 borradas de la sesion de la noche; buena parte es comentario y KDoc de por que. No se cuentan las 6 del AndroidManifest ni las de los DEVLOG.   22 DE SEPTIEMBRE: BC-14 (bloque nuevo) = el LED de estado pasa a ser tambien indicador de bateria, pedido por el cliente ese dia. No caben las dos senales en un LED y el nodo no tiene verde ni azul parpadeando, asi que el cliente decidio el reparto: el estado manda (grabando rojo parpadeo, emitiendo amarillo parpadeo) salvo por debajo del 40 %, que se impone a todo. Se sacrifica el azul de anillo armado, que solo queda en la pantalla y en el STATUS del telefono; el protocolo con el movil no cambia. PENDIENTE DE VER EN LA UNIDAD: no habia bodycam conectada, la app solo compila, y el rojo fijo usa el valor 6 del nodo, de la franja 1-6 que nunca se ha comprobado a mano. Las 1,5 h las indico el usuario. Lineas .kt sin commitear, medidas con git: 166 anadidas y 24 borradas en cuatro ficheros; buena parte es KDoc del porque del reparto de colores.   24 DE SEPTIEMBRE, ANULADO: la fila 54 (BC-15, asistente de instalacion y perfil de dispositivo, 3 h, commit cb6a247) queda TACHADA y NO se contabiliza, por decision del usuario el 28-sep: se volvio a la version estandar sin el asistente, que queda aparcado en la rama dev_install_assistant. Se vaciaron fecha, app, bloque y horas de esa fila para que las formulas no cuenten ni las horas ni el dia ni el bloque; los datos originales siguen en el texto. Las 1.402 lineas de ese commit se restaron de las del mes.   28 DE SEPTIEMBRE: BC-7 y AN-3 (emparejamiento, ya existentes) = workflow 31 v2, el canal Bluetooth entre telefono y bodycam pasa a ir cifrado (ECDH efimero firmado + AES-256-GCM por linea). Hasta hoy el token de la sesion del agente, prestado a la bodycam desde el 25-sep, viajaba en claro. Modo transicion por decision del usuario: la bodycam sigue aceptando telefonos sin cifrar mientras sus anclas no casen con las CA del backend; el token ya solo va cifrado. SIN PROBAR EN APARATOS: hoy ningun telefono se acredita ante la W1. La 1 h la indico el usuario; el reparto 0,5 / 0,5 es estimacion. Lineas .kt sin commitear, medidas con git: 326 anadidas en BC (161 de CanalCifrado, nuevo; 74 en Emparejamiento y 91 en BtServerService) y unas 426 en AN (161 de CanalCifrado, 64 en EmparejamientoBodycam, 135 de pruebas JVM y unas 66 en BodycamRepository; esta ultima es estimacion, porque el fichero lleva tambien cambios sin commitear de otra sesion).   RANGO AMPLIADO el 28-sep de la fila 55 a la 65: total en la 66 y esta leyenda en la 68. FILAS LIBRES: 57-65; al agotarlas hay que ampliar $65 en D66, K8, L5-L8 y N5-N7.</t>
+          <t>AN-2 = identidad, credencial, PIN y sesión (workflows 12, 3, 4, 27). AN-3 y BC-7 = emparejamiento y atadura con la bodycam (13, 31, 33, 34). AN-4 y BC-8 = PTT por Agora (voz de la bodycam a todos los teléfonos, y PTT propio del teléfono). AN-5 = gafas BleeqUp (enlace BT y análisis de viabilidad).   ORIGEN DE LAS HORAS: las del 4, el 6 y el 8 de septiembre salen del reloj de sesión o de marcas de fichero; el reparto por tarea dentro del 6 y el reparto por app del 8 son estimaciones sobre un total medido. La fila del 3 de septiembre está ESTIMADA y hay que confirmarla antes de facturar. El 8 de septiembre no cuenta el hueco 16:39-17:40. Las cuatro filas de desarrollo del 9 de septiembre salen de las marcas de fichero de la sesion (08:41-12:21, 3,7 h medidas) y su reparto por tarea es una estimacion; la hora de reunion de ese dia la indico el usuario y va sin bloque, como las reuniones de agosto. La fila de la tarde del 9 (gafas, 1,3 h) sale del reloj de sesion 21:05-22:25. Las 3 h del 7 de septiembre las indicó el usuario; las marcas de fichero de ese día van de 21:05 a 23:02.   LÍNEAS DE CÓDIGO: líneas .kt añadidas en el mes, medidas con git (commits del 4, 6, 8 y 9, mas el armazon de las gafas y la integracion del SDK del 9, ambos sin commitear; más el armazón de las gafas del 9, todavía sin commitear).   11 DE SEPTIEMBRE: AN-6 y BC-9 = video original a 1080p sin recodificar, proxy de 720p/15 para el LLM del backend y aviso del SOS para Agora Cloud Recording. Las dos filas salen del reloj de sesion 14:26-16:30 (2,1 h medidas) redondeado al alza a 3 h por indicacion del usuario; el reparto 1,8 AN / 1,2 BC es estimacion. Lineas del 11, sin commitear: 462 en BC medidas con git y ficheros nuevos; unas 1.169 en AN, de ellas ~80 estimadas en tres ficheros que ya traian cambios de antes.   12 DE SEPTIEMBRE: AN-5 = mando a distancia de las gafas (grabar, parar y foto por BLE). Las 3 h las indico el usuario. Lineas del 12, sin commitear: 975 anadidas medidas con git, de las cuales unas 110 no son codigo nuevo sino movido de otros ficheros (el puente del SDK sale de GafasApPrueba y el boton de accion sale del controlador de la bodycam), asi que lo genuinamente nuevo son unas 865.   REGLA DE REDONDEO (desde el 13-sep, indicada por el usuario): las horas se redondean SIEMPRE AL ALZA al medio punto. 2,7 medidas se imputan como 3; 2,1 como 2,5; 2,5 se queda en 2,5. Las filas anteriores al 13-sep se dejan como estaban.   TARDE DEL 9 DE SEPTIEMBRE (anadida el 13-sep): AN-7 = boveda, categorizacion de evidencia en bruto de los perifericos. Esta sesion NO estaba en el libro: las cuatro filas de desarrollo del 9 salen de las marcas 08:41-12:21 y la de las gafas del reloj 21:05-22:25, y esta cae en medio. Las marcas de fichero la situan entre 13:13 y 15:57 (2,7 h medidas), redondeadas al alza a 3 h. Fue a parar al commit 22768a9, que arrastra tambien el trabajo del 11. Lineas: 476 anadidas medidas con git en los cuatro ficheros que son solo de esta sesion (RawEvidenceEntities, RawEvidenceRepository, CategorizeDialog e IncidentDao). Hay otras 325 en IncidentRepository, IncidentDatabase, VaultScreen y VaultViewModel que NO se suman aqui porque podrian estar ya contadas en las filas del 11.   13 DE SEPTIEMBRE: AN-8 = rele de la bodycam a las gafas FalconOne, mas repaso de interfaz. El oficial pulsa grabar o el SOS del pecho y las gafas graban solas; el telefono hace de puente porque las gafas solo entienden el SDK del fabricante, que corre en Android. Incluye canal BLE permanente, estado de grabacion honesto, aviso de video pendiente, descarga por WiFi hasta la boveda cifrada, aviso sonoro si un SOS se queda sin gafas, textos en ingles, barra superior unificada con el patron de Android, renombrado a FalconOne y arreglos de la revision (boveda que reventaba al abrirse, nombres de fichero que se pisaban, excepcion de API 28 con minSdk 26 y descarga colgada al caerse el WiFi). Verificado contra el hardware el mismo dia. Las horas salen de marcas de fichero 15:13-23:25 (8,2 h medidas) redondeadas al alza a 8,5 h segun la regla de redondeo; NO se cuenta el analisis inicial de esta propia tabla, que fue antes de la primera marca. Lineas del 13: 2.882 anadidas medidas con git sobre los cinco commits del dia; de ellas 527 son sondas de depuracion que NO van a release.   14 DE SEPTIEMBRE: AN-9 y BC-10 = enlace con la bodycam sin MAC compilada (seleccion desde la app y unidad visible 5 min al arrancar) y uid de Agora propio por bodycam. BC-8 (PTT) = medicion de la unidad escuchando el canal. Las horas salen del reloj de sesion 19:36-19:52 y 21:53-23:50 (2,2 h medidas), redondeadas al alza a 2,5 h; el reparto 1,3 AN / 0,6 + 0,6 BC es estimacion. NO se cuenta el hueco 19:52-21:34, en el que la sesion esperaba el resultado de una prueba en el Redmi y la maquina se reinicio. Lineas del 14, sin commitear, medidas con git: 638 en AN (44 de ellas de prueba JVM) y 291 en BC, de las cuales 180 son la sonda de depuracion que NO va a release.   15 DE SEPTIEMBRE: AN-4 y BC-8 (PTT). BC-8 = la bodycam escucha el canal todo el tiempo para que el PTT de los telefonos suene por su altavoz (punto 1 de los requisitos del 14-sep). AN-4 = boton de PTT del telefono de un toque, y diagnostico de que Nexus no vuelve al canal tras perder la conexion (documentado, sin arreglar). Las horas salen del reloj de sesion 12:28-13:07 (0,65 h medidas), redondeadas al alza a 1 h; el reparto 0,5 / 0,5 es estimacion sobre las marcas de fichero (BodyCamServer 12:34-12:49, Nexus 12:59-13:04). Lineas del 15, sin commitear, medidas con git: 308 anadidas en BC (de ellas 279 en LivestreamService, reescrito: salen tambien 216) y 22 en AN.   15 DE SEPTIEMBRE, TARDE: AN-4 = reconexion al canal de Agora (el telefono se quedaba fuera sin avisar). AN-2 = revision del IAM y workflows 5 (cambio de PIN) y 30 (fin de turno). AN-10 (bloque nuevo) = auditoria local, workflows 61 y 46. Las horas salen del reloj de sesion 13:34-14:05 y 14:22-15:06 (1,25 h medidas), redondeadas al alza a 1,5 h; el reparto 0,3 / 0,6 / 0,6 es estimacion sobre la hora de cada peticion. NO se cuentan 13:20-13:34, que fue anotar en esta tabla las horas de la manana, ni 14:05-14:22, espera a que se desbloqueara el telefono de pruebas. Lineas .kt: 176 de la reconexion (commit 49d8c20, sin las 22 del boton de PTT ya contadas en la fila 33); unas 529 de los wf 5 y 30 y unas 903 de los wf 61 y 46, de ellas 96 de pruebas JVM, sin commitear; el reparto entre bloques de los ficheros compartidos (IdentityRepository, ProfileScreen, AppNavHost, AppContainer) es estimacion.   15 DE SEPTIEMBRE, FINAL DE LA TARDE: AN-5 (gafas) = selector de gafas sin MAC compilada, y arreglo de la conexion en Android 11 (el SDK del fabricante comprobaba un permiso que en esa version no existe). Las 2 h las indico el usuario; la sesion registra 0,85 h activas (15:06-15:27, 16:03-16:26 y 16:41-16:48) y los huecos 15:27-16:03 y 16:26-16:41 fueron del usuario con la release del manager y las pruebas en el Redmi. Reparto 1 / 1 estimado. Lineas .kt sin commitear, medidas con git: 378 (unas 343 del selector y unas 35 del arreglo de Android 11).   15 DE SEPTIEMBRE, NOCHE: AN-4 (PTT) = aviso de PTT pisado, con tono de tres pitidos y boton ambar cuando dos agentes hablan a la vez. La hora la indico el usuario. Lineas .kt sin commitear, medidas con git: 126 en AN (19 del atajo de debug) y 11 en BC (el tono gemelo en PttTones).   RANGO DE FORMULAS: ampliado el 14-sep de la fila 29 a la 33 y el 15-sep a la 43; el total esta en la fila 44 y esta leyenda en la 46. El 18-sep se amplio a la 55: total en la 56 y esta leyenda en la 58. Libres las filas 49-55. Al volver a ampliar, cambiar $55 en D56 y en K8, L5-L8 y N5-N7.   16 Y 17 DE SEPTIEMBRE, BACKEND (aplicacion NX, nueva): NX es el tercer repositorio, aeria-nexus, que hasta hoy no estaba en este libro aunque llevaba dos dias de trabajo. Django 5 + DRF + Celery y el panel Next.js, mas el repositorio de contratos aeria-contracts, que se imputa aqui porque nacio dentro de estas mismas sesiones. NX-1 = contratos, simulador de cliente, costuras de portabilidad e identidad F1-F6. NX-2 = ingesta de evidencia por tus y enlace de la subida con el analisis. NX-3 = coste medido, arreglos y puesta a punto para la demostracion al manager.   ORIGEN DE LAS HORAS DEL BACKEND: las dos filas del 16 salen de las marcas de los commits, 15:32 (primer commit de contratos) a 23:42 (ultimo del backend), 8,15 h medidas; el corte entre NX-1 y NX-2 es el commit de las 18:47, que cierra identidad. Cada tramo se redondea al alza al medio punto por separado (3,25-&gt;3,5 y 4,9-&gt;5), asi que la suma imputada del dia es 8,5. NO se cuenta nada anterior al primer commit. Las 2,5 h del 17 las indico el usuario: esa sesion no dejo commits, se prolongo pasada la medianoche y se imputa entera al 17.   LINEAS DE CODIGO DEL BACKEND: 10.475, medidas con git y contando solo codigo (.py, .ts, .tsx). Del 16 son 9.871 en diez commits; del 17, 604 sin commitear (469 de cuatro ficheros nuevos y 135 de modificaciones). NO se cuentan 2.210 lineas de documentacion en Markdown de los dos dias, ni las 1.028 del simulador de cliente y 456 del OpenAPI que viven en aeria-contracts, aunque se escribieran en estas sesiones: quedan anotadas aqui por si se decide sumarlas.   18 DE SEPTIEMBRE: NX-4 (bloque nuevo) = evidencia del telefono en el backend y el panel. AN-11 (bloque nuevo) = conexion de la app con el backend (IAM real, sesion, subida autenticada, manifiesto y ubicacion). NX-1 y NX-3 se reutilizan para el acceso al panel y los arreglos del panel de la manana.   ORIGEN DE LAS HORAS DEL 18: el total de 4 h lo indico el usuario. El reloj de la sesion de backend va de 10:15:48 a 14:28:12 (4,21 h) y la sesion de la app siguio hasta las 15:25; las marcas de fichero (10:58, 11:23, 12:27, 13:40) lo corroboran. El reparto 0,8 / 0,4 / 1,3 / 1,5 entre los tramos A, B y C (backend y app) es estimacion sobre ese total.   LINEAS DEL 18, sin commitear: NX 833 medidas con git sin documentacion (tramo A +209, B +105 y C +519); AN 933 (511 en ficheros existentes y 422 en nuevos). NO se cuentan las 121 lineas de documentacion de aeria-contracts.   18 DE SEPTIEMBRE, BODYCAM: BC-11 (bloque nuevo) = modo noche automatico de la W1 (LEDs IR, filtro IR-CUT, sensor de luz y blanco y negro en grabacion y SOS). Las horas salen de las marcas de fichero y del reloj de sesion 15:21-16:42 (1,35 h medidas), redondeadas al alza a 1,5 h; incluyen las dos pruebas en la unidad. Lineas .kt sin commitear, medidas con git: 310 en BC (253 en ModoNoche y MonocromoSos, nuevos, y 57 en modificaciones). El SOS en monocromo compila y esta instalado, pero queda pendiente de probar con la unidad.   20 DE SEPTIEMBRE: BC-12 (bloque nuevo) = modo kiosco de la unidad con device owner, en la rama dev_device_owner, mas el analisis de las tres vias de control y el destripado de la APK del fabricante. BC-13 y AN-12 (bloques nuevos) = cancelar desde el movil la subida de un incidente, que hasta hoy no se podia parar nunca. Las 3 h del dia las indico el usuario; el reparto 1,5 / 0,5 / 1 es estimacion. NADA de lo de hoy se ha probado en aparatos: no habia ni bodycam ni telefono conectados, las dos apps solo compilan. Lineas .kt sin commitear, medidas con git: 665 en BC (535 de tres ficheros nuevos, DeviceOwner, FalconDeviceAdmin y UploadCancel, y 130 de modificaciones) y 432 en AN (353 de dos ficheros nuevos y 79 de modificaciones); el reparto de las lineas de BC entre BC-12 y BC-13 es estimacion. NO se cuentan las lineas de tools/kiosco.sh ni las de los dos DEVLOG.   21 DE SEPTIEMBRE: BC-11 (modo noche, ya existente) = arreglo de los LEDs infrarrojos, que no se apagaban al parar de grabar, del giro de la pantalla de MainActivity y, en la sesion de la noche, del apagado de la unidad, que dejaba los infrarrojos encendidos con la bodycam apagada. Los tres fallos los observo el usuario en la unidad. Va en BC-11 y no en un bloque nuevo porque todo es corregir el modo noche entregado el 18-sep. DECISION DEL USUARIO: los IR se apagan al parar la grabacion, aunque el anillo siga armado; queda por validar con el cliente que el pre-roll nocturno de 20 s se grabe sin ellos. HORAS: las indico el usuario, que fijo la imputacion el 21-sep a las 21:00 y las subio de 1 a 1,5 h al cerrar la sesion de la noche; el trabajo se hizo entre la tarde del 20-sep y la madrugada del 21. PROBADO EN LA UNIDAD, a diferencia de lo que decia esta leyenda antes: con la bodycam por adb se midio el apagado (infrarrojo encendido 1441 lux, apagado 0) y el usuario confirmo el apagado real desde el boton. El ensayo hizo falta montarlo aparte porque ACTION_SHUTDOWN es un broadcast protegido que adb no puede enviar y la unidad es build user sin root. Medido de paso: la escritura del motor del filtro IR-CUT bloquea 2070 ms, frente a 27-44 ms de cada luz. Lineas .kt sin commitear, medidas con git: 107 anadidas y 20 borradas de la primera sesion, mas unas 230 anadidas (112 de ellas ApagadoReceiver, fichero nuevo) y 21 borradas de la sesion de la noche; buena parte es comentario y KDoc de por que. No se cuentan las 6 del AndroidManifest ni las de los DEVLOG.   22 DE SEPTIEMBRE: BC-14 (bloque nuevo) = el LED de estado pasa a ser tambien indicador de bateria, pedido por el cliente ese dia. No caben las dos senales en un LED y el nodo no tiene verde ni azul parpadeando, asi que el cliente decidio el reparto: el estado manda (grabando rojo parpadeo, emitiendo amarillo parpadeo) salvo por debajo del 40 %, que se impone a todo. Se sacrifica el azul de anillo armado, que solo queda en la pantalla y en el STATUS del telefono; el protocolo con el movil no cambia. PENDIENTE DE VER EN LA UNIDAD: no habia bodycam conectada, la app solo compila, y el rojo fijo usa el valor 6 del nodo, de la franja 1-6 que nunca se ha comprobado a mano. Las 1,5 h las indico el usuario. Lineas .kt sin commitear, medidas con git: 166 anadidas y 24 borradas en cuatro ficheros; buena parte es KDoc del porque del reparto de colores.   24 DE SEPTIEMBRE, ANULADO: la fila 54 (BC-15, asistente de instalacion y perfil de dispositivo, 3 h, commit cb6a247) queda TACHADA y NO se contabiliza, por decision del usuario el 28-sep: se volvio a la version estandar sin el asistente, que queda aparcado en la rama dev_install_assistant. Se vaciaron fecha, app, bloque y horas de esa fila para que las formulas no cuenten ni las horas ni el dia ni el bloque; los datos originales siguen en el texto. Las 1.402 lineas de ese commit se restaron de las del mes.   28 DE SEPTIEMBRE: BC-7 y AN-3 (emparejamiento, ya existentes) = workflow 31 v2, el canal Bluetooth entre telefono y bodycam pasa a ir cifrado (ECDH efimero firmado + AES-256-GCM por linea). Hasta hoy el token de la sesion del agente, prestado a la bodycam desde el 25-sep, viajaba en claro. Modo transicion por decision del usuario: la bodycam sigue aceptando telefonos sin cifrar mientras sus anclas no casen con las CA del backend; el token ya solo va cifrado. SIN PROBAR EN APARATOS: hoy ningun telefono se acredita ante la W1. La 1 h la indico el usuario; el reparto 0,5 / 0,5 es estimacion. Lineas .kt sin commitear, medidas con git: 326 anadidas en BC (161 de CanalCifrado, nuevo; 74 en Emparejamiento y 91 en BtServerService) y unas 426 en AN (161 de CanalCifrado, 64 en EmparejamientoBodycam, 135 de pruebas JVM y unas 66 en BodycamRepository; esta ultima es estimacion, porque el fichero lleva tambien cambios sin commitear de otra sesion).   RANGO AMPLIADO el 28-sep de la fila 55 a la 65: total en la 66 y esta leyenda en la 68. FILAS LIBRES: 57-65; al agotarlas hay que ampliar $65 en D66, K8, L5-L8 y N5-N7.   28 DE SEPTIEMBRE, NOCHE (sesiones en paralelo BC y AN, filas 57-60): BC-7 = BWC derivado del serial y alta de la W1 en el IAM, probada en la unidad. BC-16 (bloque nuevo) = alta de aparatos a distancia y version piloto sin identidad para el manager. AN-2 = AN-0 (ancla de perifericos del alta) y wf 53 (caducidad de la credencial). AN-4 = PTT en el directo del SOS. ORIGEN: BC, reloj de su sesion 23:25-00:20 (0,9 h) partido en 0,55 + 0,4 y redondeado al alza a 0,5 + 0,5; AN, marcas de fichero 23:20-23:55 (0,6 h) que dio la propia sesion AN, redondeadas al alza a 1 h y repartidas 0,5 / 0,5 por estimacion. LINEAS .kt medidas con git: BC 94 (74 en el commit 58493ba sin contar UploadService, que es del 28 por la tarde, y 20 sin commitear); no se cuentan las 265 del guion tools/alta-bodycam-iam.sh. AN unas 596 (181 en el commit 2516769, 114 modificadas y 301 en ficheros nuevos sin commitear del wf 53, pruebas JVM incluidas). FILAS LIBRES: 62-65.   29 DE SEPTIEMBRE (fila 61): AN-13 (bloque nuevo) = SOS con directo: circulo del mapa que abre el directo, silencios locales de emisor y receptor, micro del emisor conmutable y tono de SOS configurable. ORIGEN: 2,5 h indicadas por el usuario; el reloj de la sesion daba ~0,95 h (13:10-13:55 con el inicio estimado, y 14:58-15:10 de pruebas en aparato), y el resto es su tiempo instalando y probando. La parte de la bodycam (tono, doble F2, micro en SOS) la hizo la sesion BC y va aparte. LINEAS .kt sin commitear, medidas con git: unas 800 en AN (458 en cinco ficheros nuevos; unas 90 son el boton PTT movido de Operations, no codigo nuevo).</t>
         </is>
       </c>
       <c r="J68" s="2" t="n"/>

</xml_diff>

<commit_message>
alta agente con qr, suspecion de agente, base cifrada, mapa aviso sos remoto
</commit_message>
<xml_diff>
--- a/tabla_horas_facturacion_proyecto.xlsx
+++ b/tabla_horas_facturacion_proyecto.xlsx
@@ -34971,7 +34971,7 @@
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>BC-17</t>
+          <t>BC-17, BC-18</t>
         </is>
       </c>
       <c r="L5" s="13">
@@ -34979,7 +34979,7 @@
         <v/>
       </c>
       <c r="M5" s="13" t="n">
-        <v>1211</v>
+        <v>1401</v>
       </c>
       <c r="N5" s="13">
         <f>SUMIFS($D$4:$D$65,$B$4:$B$65,"BC",$G$4:$G$65,"&lt;&gt;Sí")</f>
@@ -34990,7 +34990,7 @@
         <v/>
       </c>
     </row>
-    <row r="6">
+    <row r="6" s="15">
       <c r="A6" s="18" t="n">
         <v>46298</v>
       </c>
@@ -35034,7 +35034,7 @@
       </c>
       <c r="K6" s="11" t="inlineStr">
         <is>
-          <t>AN-14</t>
+          <t>AN-14, AN-15, AN-16</t>
         </is>
       </c>
       <c r="L6" s="13">
@@ -35042,7 +35042,7 @@
         <v/>
       </c>
       <c r="M6" s="13" t="n">
-        <v>398</v>
+        <v>1880</v>
       </c>
       <c r="N6" s="13">
         <f>SUMIFS($D$4:$D$65,$B$4:$B$65,"AN",$G$4:$G$65,"&lt;&gt;Sí")</f>
@@ -35053,15 +35053,43 @@
         <v/>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="18" t="n"/>
-      <c r="B7" s="19" t="n"/>
-      <c r="C7" s="19" t="n"/>
-      <c r="D7" s="19" t="n"/>
-      <c r="E7" s="19" t="n"/>
-      <c r="F7" s="19" t="n"/>
-      <c r="G7" s="19" t="n"/>
-      <c r="H7" s="19" t="n"/>
+    <row r="7" s="15">
+      <c r="A7" s="18" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>BC-18</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Subida rechazada por la credencial y coordinacion con backend y movil por las altas desde el panel y la suspension de perfiles (rama dev_whisper_text). Revision de la unidad contra iam-session.md: no mira roles ni alcances. ChunkedUploader lee el motivo de un 401/403 (cabecera X-Error-Code o code del cuerpo), corta sin reintentos y suelta el token prestado salvo insufficient_scope; lo pendiente espera a un token nuevo. Motivo al telefono por BT: UPLOAD_REJECTED y campo rejected en UPLOAD_LIST. Clave nueva officer_user_id en Upload-Metadata (quien grabo) para que el backend deje de atribuir por la sesion que sube. El token sobrevive a la caida del Bluetooth y se retira al acreditarse otro telefono. Contrato escrito en aeria-contracts/upload-protocol.md 5.3 y docs/UPLOAD-PROTOCOL.md. COMPILA; SIN PROBAR EN LA W1 NI CONTRA EL BACKEND</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>2 h</t>
+        </is>
+      </c>
       <c r="J7" s="13" t="inlineStr">
         <is>
           <t>aeria-nexus (backend)</t>
@@ -35069,7 +35097,7 @@
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>NX-5</t>
+          <t>NX-5, NX-6, NX-7, NX-8, NX-9, NX-10, NX-11, NX-12, NX-13, NX-14</t>
         </is>
       </c>
       <c r="L7" s="13">
@@ -35077,7 +35105,7 @@
         <v/>
       </c>
       <c r="M7" s="13" t="n">
-        <v>92</v>
+        <v>8217</v>
       </c>
       <c r="N7" s="13">
         <f>SUMIFS($D$4:$D$65,$B$4:$B$65,"NX",$G$4:$G$65,"&lt;&gt;Sí")</f>
@@ -35088,15 +35116,43 @@
         <v/>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="18" t="n"/>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="19" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="19" t="n"/>
-      <c r="F8" s="19" t="n"/>
-      <c r="G8" s="19" t="n"/>
-      <c r="H8" s="19" t="n"/>
+    <row r="8" s="15">
+      <c r="A8" s="18" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C8" s="19" t="inlineStr">
+        <is>
+          <t>NX-6</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
+        <is>
+          <t>Tres niveles de usuario y altas desde el panel (rama dev_whisper_text de aeria-nexus). superadmin / admin / user como paquetes de los siete roles IAM, que no se tocan. Endpoints /api/users/ (alta, cambio de nivel, suspension, acceso al panel con TOTP) y pantalla /users con codigo QR; el menu ensena a quien ha entrado. Arreglado el CSRF del panel: ningun POST funcionaba en el navegador. Codigos de error estables en los 401/403 (cuerpo y cabecera X-Error-Code). El backend entrega nombre, rango y placa al telefono (profile en sesion y enrolamiento). Atribucion de la evidencia a quien la grabo (officer_user_id, NOAGENT) y piezas de un incidente atadas entre telefonos distintos. Endpoints de SOS (start, heartbeat, stop), que daban 404, y sesion restringida sos_only para que el SOS de un agente suspendido llegue; sin grabacion en la nube de Agora. Coordinacion y revision de las sesiones del movil y de la bodycam contra iam-session.md; contrato en aeria-contracts (iam-session 3.1, 5.7, 5.8, 6 y 9; upload-protocol 5.1 y 5.2). Migraciones 0017 y 0018. 333 tests en verde, 53 nuevos. LA PANTALLA /users NO SE HA ABIERTO EN UN NAVEGADOR; nada probado con dispositivos reales</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H8" s="19" t="inlineStr">
+        <is>
+          <t>2 h</t>
+        </is>
+      </c>
       <c r="J8" s="10" t="inlineStr">
         <is>
           <t>TOTAL DEL MES</t>
@@ -35123,15 +35179,43 @@
         <v/>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="18" t="n"/>
-      <c r="B9" s="19" t="n"/>
-      <c r="C9" s="19" t="n"/>
-      <c r="D9" s="19" t="n"/>
-      <c r="E9" s="19" t="n"/>
-      <c r="F9" s="19" t="n"/>
-      <c r="G9" s="19" t="n"/>
-      <c r="H9" s="19" t="n"/>
+    <row r="9" s="15">
+      <c r="A9" s="18" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>AN-15</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="19" t="inlineStr">
+        <is>
+          <t>Altas desde el panel, perfil del agente y suspension de perfiles en el telefono (rama dev_back_connection). Revision del telefono contra iam-session.md y coordinacion con las sesiones del backend y de la bodycam: no mira roles ni alcances; se corrigen en el contrato la declaracion de la atadura y cuatro frases que no describian al telefono. Alta del agente: el identificador se teclea entero (formulario OFFICER ID, minusculas, sin espacios, misma regla que el panel) en vez de ir fijo en el codigo. Mensajes propios en ingles segun el code del backend (perfil suspendido, revocado, inexistente, telefono no reconocido). Nombre, rango y placa llegan del backend en el alta y en cada sesion, se guardan en el telefono y son los que firma la atadura con la bodycam. Agente suspendido o revocado a mitad de turno: se deja de reintentar, se descarta el token, se avisa al agente y sigue grabando en local; CHECK AGAIN o el siguiente desbloqueo vuelven a preguntar. Sesion restringida sos_only para que el SOS de un suspendido llegue al backend, prestada tambien a la bodycam. COMPILA Y PASAN LOS TESTS DE UNIDAD; SIN PROBAR EN APARATO NI CONTRA EL BACKEND</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
+        <is>
+          <t>2 h</t>
+        </is>
+      </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
           <t>Tarifa (€/h)</t>
@@ -35146,14 +35230,42 @@
       <c r="O9" s="2" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n"/>
-      <c r="B10" s="19" t="n"/>
-      <c r="C10" s="19" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
+      <c r="A10" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C10" s="19" t="inlineStr">
+        <is>
+          <t>NX-6</t>
+        </is>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E10" s="19" t="inlineStr">
+        <is>
+          <t>Ajustes del alta tras la respuesta de las dos apps (rama dev_whisper_text): reintento idempotente del enrolamiento del agente, codigos en el 409 del alta de dispositivo, emparejamientos con caducidad en milisegundos y el fin de turno suelta la camara en la misma peticion</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>7effe73, 498cd98</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H10" s="19" t="inlineStr">
+        <is>
+          <t>reloj de sesion 0,3 h</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="n"/>
       <c r="K10" s="2" t="n"/>
       <c r="L10" s="2" t="n"/>
@@ -35162,14 +35274,42 @@
       <c r="O10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="18" t="n"/>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="19" t="n"/>
-      <c r="D11" s="19" t="n"/>
-      <c r="E11" s="19" t="n"/>
-      <c r="F11" s="19" t="n"/>
-      <c r="G11" s="19" t="n"/>
-      <c r="H11" s="19" t="n"/>
+      <c r="A11" s="18" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr">
+        <is>
+          <t>NX-6</t>
+        </is>
+      </c>
+      <c r="D11" s="19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="19" t="inlineStr">
+        <is>
+          <t>Primera vez que el panel se abre en el navegador: boton de salir, Users visible para el superadmin, rango como desplegable obligatorio, nombre y apellidos en dos campos y cuentas personales en local</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>d766513, f2ae93e</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H11" s="19" t="inlineStr">
+        <is>
+          <t>reloj de sesion 1,2 h</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="n"/>
       <c r="K11" s="2" t="n"/>
       <c r="L11" s="2" t="n"/>
@@ -35178,14 +35318,42 @@
       <c r="O11" s="2" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n"/>
-      <c r="B12" s="19" t="n"/>
-      <c r="C12" s="19" t="n"/>
-      <c r="D12" s="19" t="n"/>
-      <c r="E12" s="19" t="n"/>
-      <c r="F12" s="19" t="n"/>
-      <c r="G12" s="19" t="n"/>
-      <c r="H12" s="19" t="n"/>
+      <c r="A12" s="18" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B12" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C12" s="19" t="inlineStr">
+        <is>
+          <t>NX-7</t>
+        </is>
+      </c>
+      <c r="D12" s="19" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E12" s="19" t="inlineStr">
+        <is>
+          <t>Documento de aclaracion IAM contrastado con los Excel IAM y con las dos apps; informe de contradicciones para el manager, en espanol y en ingles (docs/)</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H12" s="19" t="inlineStr">
+        <is>
+          <t>reloj de sesion 0,4 h</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="n"/>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
@@ -35194,14 +35362,42 @@
       <c r="O12" s="2" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="18" t="n"/>
-      <c r="B13" s="19" t="n"/>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
-      <c r="G13" s="19" t="n"/>
-      <c r="H13" s="19" t="n"/>
+      <c r="A13" s="18" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B13" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>NX-8</t>
+        </is>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="19" t="inlineStr">
+        <is>
+          <t>Workflows del piloto en el backend: recibo de aceptacion firmado, desfase de reloj del dispositivo, rechazo de unidades revocadas o no enroladas, version minima de la app y auditoria con cadena de hashes</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>5858d8f</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H13" s="19" t="inlineStr">
+        <is>
+          <t>reloj de sesion 1 h</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
@@ -35210,14 +35406,42 @@
       <c r="O13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n"/>
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="19" t="n"/>
-      <c r="D14" s="19" t="n"/>
-      <c r="E14" s="19" t="n"/>
-      <c r="F14" s="19" t="n"/>
-      <c r="G14" s="19" t="n"/>
-      <c r="H14" s="19" t="n"/>
+      <c r="A14" s="18" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B14" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C14" s="19" t="inlineStr">
+        <is>
+          <t>NX-9</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="19" t="inlineStr">
+        <is>
+          <t>Seguridad: todo exige sesion por defecto (con test que recorre todas las rutas), /media cerrado, cache de evidencia en claro de vida corta, enrolamiento rechaza identidades revocadas y atribucion por binding_id</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>a96a4ce</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H14" s="19" t="inlineStr">
+        <is>
+          <t>reloj de sesion 0,8 h</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
@@ -35226,14 +35450,42 @@
       <c r="O14" s="2" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="n"/>
-      <c r="B15" s="19" t="n"/>
-      <c r="C15" s="19" t="n"/>
-      <c r="D15" s="19" t="n"/>
-      <c r="E15" s="19" t="n"/>
-      <c r="F15" s="19" t="n"/>
-      <c r="G15" s="19" t="n"/>
-      <c r="H15" s="19" t="n"/>
+      <c r="A15" s="18" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B15" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>NX-10</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="19" t="inlineStr">
+        <is>
+          <t>Panel: pantallas de auditoria, cadena de custodia del incidente y dispositivos; nuevo alta de camaras con permiso de un solo uso y revocaciones que se levantan</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>f2ae93e</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>reloj de sesion 1 h</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="n"/>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
@@ -35242,14 +35494,42 @@
       <c r="O15" s="2" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n"/>
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-      <c r="E16" s="19" t="n"/>
-      <c r="F16" s="19" t="n"/>
-      <c r="G16" s="19" t="n"/>
-      <c r="H16" s="19" t="n"/>
+      <c r="A16" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="inlineStr">
+        <is>
+          <t>NX-11</t>
+        </is>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>SOS en directo en el panel por Agora: endpoint de SOS en curso, pagina /sos, aviso en todas las pantallas y visor como espectador; prueba completa con un telefono real contra el backend local</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
+        <is>
+          <t>3 h</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="n"/>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
@@ -35258,14 +35538,40 @@
       <c r="O16" s="2" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="18" t="n"/>
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="19" t="n"/>
+      <c r="A17" s="18" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>NX-12</t>
+        </is>
+      </c>
       <c r="D17" s="19" t="n"/>
-      <c r="E17" s="19" t="n"/>
-      <c r="F17" s="19" t="n"/>
-      <c r="G17" s="19" t="n"/>
-      <c r="H17" s="19" t="n"/>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>Alta por QR desde el panel (propuesta revisada con la sesion del telefono, backend y panel) y guia de alta en Word. Sin terminar</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H17" s="19" t="inlineStr">
+        <is>
+          <t>pendiente: se fija al terminar</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
@@ -35273,15 +35579,43 @@
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
     </row>
-    <row r="18">
-      <c r="A18" s="18" t="n"/>
-      <c r="B18" s="19" t="n"/>
-      <c r="C18" s="19" t="n"/>
-      <c r="D18" s="19" t="n"/>
-      <c r="E18" s="19" t="n"/>
-      <c r="F18" s="19" t="n"/>
-      <c r="G18" s="19" t="n"/>
-      <c r="H18" s="19" t="n"/>
+    <row r="18" s="15">
+      <c r="A18" s="18" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>AN</t>
+        </is>
+      </c>
+      <c r="C18" s="19" t="inlineStr">
+        <is>
+          <t>AN-16</t>
+        </is>
+      </c>
+      <c r="D18" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>Avisos SOS del mapa que no desaparecian e historial de SOS (rama dev_back_connection). Diagnostico: el banner y el tooltip del SOS de otro agente solo se quitaban con su cancelacion, que se pierde si el emisor se queda sin red, se le cierra la app o se apaga; el aviso "Signal cut" no caduca nunca y el marcador gris "Last seen" solo se borra si el agente sale del canal de forma ordenada. Ahora un SOS del que no se oye nada en 10 s se da por cortado (tambien si el emisor sale del canal), con la hora de su ultima senal. Boton de cerrar en el banner del SOS y en el marcador "Last seen". Boton de aviso junto al de centrar con contador del total de SOS y lista de todos los SOS registrados (agente, origen, fecha, inicio y fin), solo lectura, leida del backend (GET sos) con copia local si no hay conexion. El telefono que lleva la bodycam avisa al backend de su SOS (inicio, latidos y fin), que antes no quedaba registrado. Coordinado con la sesion del backend (contrato aeria-contracts sos-and-proxy.md 2.6). COMPILA Y PASAN LOS TESTS DE UNIDAD; SIN PROBAR EN APARATO</t>
+        </is>
+      </c>
+      <c r="F18" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H18" s="19" t="inlineStr">
+        <is>
+          <t>2 h</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="n"/>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
@@ -35290,14 +35624,42 @@
       <c r="O18" s="2" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="18" t="n"/>
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
-      <c r="E19" s="19" t="n"/>
-      <c r="F19" s="19" t="n"/>
-      <c r="G19" s="19" t="n"/>
-      <c r="H19" s="19" t="n"/>
+      <c r="A19" s="18" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>NX-13</t>
+        </is>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="19" t="inlineStr">
+        <is>
+          <t>Cifrado y seguridad a partir de los requisitos del manager (Security Feature List). Informe para el tecnico de ciberseguridad en espanol y en ingles (docs/, 4 paginas cada uno): matriz dato por lugar, comunicaciones, IAM, algoritmos, identidad del agente en la evidencia y requisitos frente a lo construido. Arreglos en el backend: la copia descifrada que se sube a Azure Video Indexer se borra al indexar (y comando purge_video_indexer para lo anterior); semilla TOTP de los supervisores cifrada en la base (AES-256-GCM, FIELD_ENCRYPTION_KEY, migracion 0025); HTTPS con TLS 1.2/1.3, HSTS y cookies Secure detras de nginx; manifiesto cifrado (.fev) y fotos de la unidad como incidente propio. Contratos en aeria-contracts: transport.md nuevo (TLS y pinning del telefono), manifiesto cifrado, fotos de la unidad y officer_code. Encargos de cifrado a la bodycam y al telefono, revisados punto a punto. 491 tests en verde. NADA PROBADO EN APARATO NI EN EL ENTORNO CON AZURE</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>sin commitear</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H19" s="19" t="inlineStr">
+        <is>
+          <t>3 h</t>
+        </is>
+      </c>
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n"/>
@@ -35306,14 +35668,42 @@
       <c r="O19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n"/>
-      <c r="B20" s="19" t="n"/>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="19" t="n"/>
-      <c r="G20" s="19" t="n"/>
-      <c r="H20" s="19" t="n"/>
+      <c r="A20" s="18" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>NX</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>NX-14</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="19" t="inlineStr">
+        <is>
+          <t>Puesta en marcha del servidor de Azure (nexus.aeriaone.com) con la version nueva: superadmin creado en el servidor, revision de la configuracion desplegada, Agora para el SOS en directo, direccion del servidor en el QR de alta y autoridades de certificados creadas. Diagnostico con la sesion del telefono del alta por QR contra el servidor: error 500 propio de PostgreSQL al bloquear el perfil del agente (no aparecia con SQLite en local); arreglado. Detectados para la tanda de seguridad: DEBUG activo en el servidor, cuenta demo y clave de evidencia pendiente. 491 tests en verde</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>ff3c6d1</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H20" s="19" t="inlineStr">
+        <is>
+          <t>3 h</t>
+        </is>
+      </c>
       <c r="J20" s="2" t="n"/>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
@@ -36083,7 +36473,7 @@
     <row r="68" ht="57.75" customHeight="1" s="15">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>OCTUBRE 2026. Misma estructura que septiembre: sesiones en A4:H65, total en D66, filas libres 6-65.   BLOQUES NUEVOS: BC-17 = transcripcion del audio de la evidencia con Whisper en la bodycam. NX-5 = el backend recibe la transcripcion (kind=transcript) y contrato en aeria-contracts.   2 DE OCTUBRE: 2,5 h indicadas por el usuario para la sesion; el reparto 2 / 0,5 entre BC y NX es estimacion (el trabajo de backend fue la ultima media hora). La parte de la app del telefono (transcripcion en el movil y recepcion de la de la bodycam) la hizo la sesion AN y NO esta en estas 2,5 h.   LINEAS DE CODIGO DEL 2-oct, sin commitear, medidas con git: BC 1.211 (339 en ficheros existentes y 872 en cinco nuevos: AudioPcm, Transcriber, WhisperNative, whisper_jni.cpp y CMakeLists); NO se cuentan las ~6,6 MB de whisper.cpp copiadas tal cual ni el modelo de 32 MB. NX 92 (69 en .py modificados, de ellos ~45 de tests, y 23 de la migracion); no se cuentan las ~190 lineas de transcript-format.md ni el resto de documentacion.   AN-14 = reinicio de la boveda de evidencia con el PIN cuando se olvida la contrasena.   3 DE OCTUBRE: 1,5 h de la sesion AN, un solo bloque.   LINEAS DE CODIGO DEL 3-oct, sin commitear: AN 398 anadidas (223 en el fichero nuevo VaultResetContent y el resto en EvidenceVault, VaultViewModel, VaultScreen, IdentityRepository, AuditoriaLocal, VaultRepository y AppNavHost); en VaultViewModel y VaultScreen se cuentan solo las de este bloque, no las de la transcripcion del 2-oct.</t>
+          <t>OCTUBRE 2026. Misma estructura que septiembre: sesiones en A4:H65, total en D66, filas libres 8-65 (8 y 9 reservadas el 9-oct para NX y AN).   BLOQUES NUEVOS: BC-17 = transcripcion del audio de la evidencia con Whisper en la bodycam. NX-5 = el backend recibe la transcripcion (kind=transcript) y contrato en aeria-contracts.   2 DE OCTUBRE: 2,5 h indicadas por el usuario para la sesion; el reparto 2 / 0,5 entre BC y NX es estimacion (el trabajo de backend fue la ultima media hora). La parte de la app del telefono (transcripcion en el movil y recepcion de la de la bodycam) la hizo la sesion AN y NO esta en estas 2,5 h.   LINEAS DE CODIGO DEL 2-oct, sin commitear, medidas con git: BC 1.211 (339 en ficheros existentes y 872 en cinco nuevos: AudioPcm, Transcriber, WhisperNative, whisper_jni.cpp y CMakeLists); NO se cuentan las ~6,6 MB de whisper.cpp copiadas tal cual ni el modelo de 32 MB. NX 92 (69 en .py modificados, de ellos ~45 de tests, y 23 de la migracion); no se cuentan las ~190 lineas de transcript-format.md ni el resto de documentacion.   AN-14 = reinicio de la boveda de evidencia con el PIN cuando se olvida la contrasena.   3 DE OCTUBRE: 1,5 h de la sesion AN, un solo bloque.   LINEAS DE CODIGO DEL 3-oct, sin commitear: AN 398 anadidas (223 en el fichero nuevo VaultResetContent y el resto en EvidenceVault, VaultViewModel, VaultScreen, IdentityRepository, AuditoriaLocal, VaultRepository y AppNavHost); en VaultViewModel y VaultScreen se cuentan solo las de este bloque, no las de la transcripcion del 2-oct.   BC-18 = subida rechazada por la credencial: motivo al telefono, sin reintentos, officer_user_id en la metadata y token que sobrevive al corte de Bluetooth.   9 DE OCTUBRE: 2 h por sesion para cada una de las tres sesiones (BC, NX y AN); cada sesion anota su fila.   LINEAS DE CODIGO DEL 9-oct en BC, sin commitear: unas 190 anadidas (98 medidas con git en ChunkedUploader y UploadConfig; el resto, en UploadService, Protocol y BtServerService, estimado porque esos ficheros llevan tambien lo del 2-oct sin commitear); no se cuenta la documentacion.   AN-15 = altas desde el panel en el telefono: identificador del agente tecleado, perfil del agente desde el backend para la atadura con la bodycam, aviso de perfil suspendido sin bloquear la app y SOS del agente suspendido.   LINEAS DE CODIGO DEL 9-oct en AN, sin commitear, medidas con git: 645 anadidas (391 en once ficheros .kt existentes y 254 en tres nuevos: PerfilDelAgente, EnrollmentAgenteForm y ProfileCutDialog); no se cuentan DEVLOG ni la documentacion.   NX-6 = tres niveles de usuario, altas desde el panel, codigos de error, atribucion de la evidencia a quien la grabo y SOS (endpoints y sesion restringida de un suspendido).   LINEAS DE CODIGO DEL 9-oct en NX, sin commitear, medidas con git: 2.556 anadidas (2.019 en nueve ficheros nuevos: iam_levels, iam_user_views, sos_models, sos_views, test_user_admin, test_sos, las migraciones 0017 y 0018 y la pagina /users del panel; 449 en ficheros existentes del backend y del panel; y 88 de test_tus, descontadas las ~45 del 2-oct que siguen sin commitear en ese fichero). De ellas, unas 800 son tests. No se cuentan package-lock.json, el DEVLOG ni la documentacion de aeria-contracts.   NX-7 = documento de aclaracion IAM contrastado e informe de contradicciones. NX-8 = workflows del piloto (recibo firmado, desfase de reloj, unidades revocadas, version minima, auditoria). NX-9 = seguridad (denegar por defecto, /media cerrado, cache en claro de vida corta, atribucion por binding_id). NX-10 = panel de auditoria, custodia y dispositivos, y nuevo alta de camaras. NX-11 = SOS en directo en el panel por Agora. NX-12 = alta por QR desde el panel y guia de alta.   10 A 19 DE OCTUBRE (NX): horas del reloj de las sesiones de Claude Code en el proyecto, sin pausas de mas de 30 min, repartidas entre bloques por la hora de commits y ficheros y redondeadas al alza al medio punto; NX-11 fijado en 3 h. NX-12 sin horas: se fija cuando se termine.   LINEAS DE CODIGO NX del 10 al 18-oct, medidas con git, sin documentacion ni package-lock.json: NX-6 262 (258 el 10-oct en 7effe73 y 498cd98, 4 el 12-oct en d766513; el resto del 12-oct entro en f2ae93e mezclado con NX-10 y se cuenta alli); NX-8 1.664 (5858d8f); NX-9 665 (a96a4ce); NX-10 1.742 (f2ae93e, incluye los ajustes del panel del 12-oct); NX-11 595, sin commitear (sos_views, test_sos, pagina /sos, SosLiveViewer, Layout y api.ts). NX-12 (~730 sin commitear) no se suma en M7 hasta fijar sus horas.   AN-16 = avisos SOS del mapa que caducan cuando el emisor deja de emitir, botones de cerrar e historial de SOS con contador leido del backend.   21 DE OCTUBRE: 2 h de la sesion AN, un solo bloque.   LINEAS DE CODIGO DEL 21-oct en AN, sin commitear: 837 anadidas (828 medidas con git: 408 en tres ficheros nuevos, HistorialSos, HistorialSosBackend y SosHistoryDialog, y 420 en AgoraRepository, MapScreen y MapViewModel; unas 9 estimadas en AppContainer, SosNotifier y AppNavHost, que llevan tambien cambios anteriores sin commitear); no se cuentan DEVLOG ni la documentacion.   NX-13 = cifrado y seguridad: informe para ciberseguridad (ES/EN), borrado de la copia en Video Indexer, semilla TOTP cifrada, HTTPS con HSTS y cookies seguras, manifiesto cifrado, contrato de transporte y encargos de cifrado a las dos apps.   25 DE OCTUBRE: 3 h de la sesion NX, un solo bloque.   LINEAS DE CODIGO DEL 25-oct en NX, sin commitear, medidas con git: 637 (382 en cuatro ficheros nuevos: fields.py, purge_video_indexer, la migracion 0025 y test_cifrado_backend; 255 en settings, azure_service, checks, models, tasks, tus_views, test_tus, requirements, .env.example y la plantilla de nginx). No se cuentan los ~730 del generador del informe en docs/fuentes-informe, el DEVLOG ni aeria-contracts.</t>
         </is>
       </c>
       <c r="J68" s="2" t="n"/>

</xml_diff>